<commit_message>
Data and version updated
</commit_message>
<xml_diff>
--- a/numbers.xlsx
+++ b/numbers.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nodir\Projects\open-budget-search\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28CAC716-B4CB-4779-9F69-75DB3CA82D84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D9C5CC6-A1EC-453D-B0F0-4B57D4E3DD28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{0AABE945-EFF0-4E0B-A9BD-4BB876D9C82D}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="966" uniqueCount="951">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1168" uniqueCount="1153">
   <si>
     <t>**-*14-63-61</t>
   </si>
@@ -2887,14 +2887,621 @@
   </si>
   <si>
     <t>**-*56-66-20</t>
+  </si>
+  <si>
+    <t>**-*71-80-85</t>
+  </si>
+  <si>
+    <t>**-*51-67-61</t>
+  </si>
+  <si>
+    <t>**-*18-60-64</t>
+  </si>
+  <si>
+    <t>**-*92-24-92</t>
+  </si>
+  <si>
+    <t>**-*05-27-03</t>
+  </si>
+  <si>
+    <t>**-*83-04-24</t>
+  </si>
+  <si>
+    <t>**-*83-01-82</t>
+  </si>
+  <si>
+    <t>**-*82-76-79</t>
+  </si>
+  <si>
+    <t>**-*74-35-85</t>
+  </si>
+  <si>
+    <t>**-*51-80-04</t>
+  </si>
+  <si>
+    <t>**-*84-84-18</t>
+  </si>
+  <si>
+    <t>**-*00-71-17</t>
+  </si>
+  <si>
+    <t>**-*70-96-19</t>
+  </si>
+  <si>
+    <t>**-*69-11-23</t>
+  </si>
+  <si>
+    <t>**-*78-91-95</t>
+  </si>
+  <si>
+    <t>**-*89-41-91</t>
+  </si>
+  <si>
+    <t>**-*74-55-66</t>
+  </si>
+  <si>
+    <t>**-*17-76-77</t>
+  </si>
+  <si>
+    <t>**-*71-33-08</t>
+  </si>
+  <si>
+    <t>**-*97-43-33</t>
+  </si>
+  <si>
+    <t>**-*89-60-61</t>
+  </si>
+  <si>
+    <t>**-*74-25-84</t>
+  </si>
+  <si>
+    <t>**-*63-78-99</t>
+  </si>
+  <si>
+    <t>**-*93-13-93</t>
+  </si>
+  <si>
+    <t>**-*81-12-61</t>
+  </si>
+  <si>
+    <t>**-*64-00-79</t>
+  </si>
+  <si>
+    <t>**-*52-86-76</t>
+  </si>
+  <si>
+    <t>**-*22-11-87</t>
+  </si>
+  <si>
+    <t>**-*56-77-02</t>
+  </si>
+  <si>
+    <t>**-*46-84-81</t>
+  </si>
+  <si>
+    <t>**-*27-88-07</t>
+  </si>
+  <si>
+    <t>**-*35-89-88</t>
+  </si>
+  <si>
+    <t>**-*46-66-03</t>
+  </si>
+  <si>
+    <t>**-*15-33-66</t>
+  </si>
+  <si>
+    <t>**-*37-00-63</t>
+  </si>
+  <si>
+    <t>**-*47-78-15</t>
+  </si>
+  <si>
+    <t>**-*82-98-00</t>
+  </si>
+  <si>
+    <t>**-*16-22-09</t>
+  </si>
+  <si>
+    <t>**-*92-51-51</t>
+  </si>
+  <si>
+    <t>**-*04-87-90</t>
+  </si>
+  <si>
+    <t>**-*61-16-25</t>
+  </si>
+  <si>
+    <t>**-*89-00-64</t>
+  </si>
+  <si>
+    <t>**-*11-37-74</t>
+  </si>
+  <si>
+    <t>**-*03-22-28</t>
+  </si>
+  <si>
+    <t>**-*89-92-12</t>
+  </si>
+  <si>
+    <t>**-*23-65-05</t>
+  </si>
+  <si>
+    <t>**-*97-92-20</t>
+  </si>
+  <si>
+    <t>**-*11-70-04</t>
+  </si>
+  <si>
+    <t>**-*27-78-78</t>
+  </si>
+  <si>
+    <t>**-*07-95-90</t>
+  </si>
+  <si>
+    <t>**-*52-09-98</t>
+  </si>
+  <si>
+    <t>**-*39-67-07</t>
+  </si>
+  <si>
+    <t>**-*26-92-29</t>
+  </si>
+  <si>
+    <t>**-*11-88-10</t>
+  </si>
+  <si>
+    <t>**-*29-92-26</t>
+  </si>
+  <si>
+    <t>**-*49-44-35</t>
+  </si>
+  <si>
+    <t>**-*73-99-03</t>
+  </si>
+  <si>
+    <t>**-*53-95-72</t>
+  </si>
+  <si>
+    <t>**-*34-95-02</t>
+  </si>
+  <si>
+    <t>**-*79-25-11</t>
+  </si>
+  <si>
+    <t>**-*16-60-33</t>
+  </si>
+  <si>
+    <t>**-*57-05-91</t>
+  </si>
+  <si>
+    <t>**-*57-26-26</t>
+  </si>
+  <si>
+    <t>**-*53-37-55</t>
+  </si>
+  <si>
+    <t>**-*02-99-59</t>
+  </si>
+  <si>
+    <t>**-*82-92-20</t>
+  </si>
+  <si>
+    <t>**-*73-29-91</t>
+  </si>
+  <si>
+    <t>**-*44-17-47</t>
+  </si>
+  <si>
+    <t>**-*42-27-59</t>
+  </si>
+  <si>
+    <t>**-*60-96-80</t>
+  </si>
+  <si>
+    <t>**-*74-03-23</t>
+  </si>
+  <si>
+    <t>**-*33-29-91</t>
+  </si>
+  <si>
+    <t>**-*17-12-55</t>
+  </si>
+  <si>
+    <t>**-*17-88-11</t>
+  </si>
+  <si>
+    <t>**-*66-20-02</t>
+  </si>
+  <si>
+    <t>**-*99-84-94</t>
+  </si>
+  <si>
+    <t>**-*78-10-69</t>
+  </si>
+  <si>
+    <t>**-*50-52-59</t>
+  </si>
+  <si>
+    <t>**-*99-94-19</t>
+  </si>
+  <si>
+    <t>**-*86-40-29</t>
+  </si>
+  <si>
+    <t>**-*15-60-88</t>
+  </si>
+  <si>
+    <t>**-*70-40-29</t>
+  </si>
+  <si>
+    <t>**-*26-84-08</t>
+  </si>
+  <si>
+    <t>**-*54-39-10</t>
+  </si>
+  <si>
+    <t>**-*05-12-78</t>
+  </si>
+  <si>
+    <t>**-*49-01-41</t>
+  </si>
+  <si>
+    <t>**-*36-24-87</t>
+  </si>
+  <si>
+    <t>**-*72-98-08</t>
+  </si>
+  <si>
+    <t>**-*77-07-99</t>
+  </si>
+  <si>
+    <t>**-*51-08-87</t>
+  </si>
+  <si>
+    <t>**-*77-49-06</t>
+  </si>
+  <si>
+    <t>**-*96-20-18</t>
+  </si>
+  <si>
+    <t>**-*40-75-73</t>
+  </si>
+  <si>
+    <t>**-*44-75-73</t>
+  </si>
+  <si>
+    <t>**-*64-02-91</t>
+  </si>
+  <si>
+    <t>**-*03-79-99</t>
+  </si>
+  <si>
+    <t>**-*32-31-60</t>
+  </si>
+  <si>
+    <t>**-*01-84-88</t>
+  </si>
+  <si>
+    <t>**-*31-56-92</t>
+  </si>
+  <si>
+    <t>**-*02-70-80</t>
+  </si>
+  <si>
+    <t>**-*09-19-83</t>
+  </si>
+  <si>
+    <t>**-*27-11-30</t>
+  </si>
+  <si>
+    <t>**-*33-08-95</t>
+  </si>
+  <si>
+    <t>**-*06-83-97</t>
+  </si>
+  <si>
+    <t>**-*04-14-66</t>
+  </si>
+  <si>
+    <t>**-*56-25-91</t>
+  </si>
+  <si>
+    <t>**-*69-17-76</t>
+  </si>
+  <si>
+    <t>**-*46-73-71</t>
+  </si>
+  <si>
+    <t>**-*16-16-82</t>
+  </si>
+  <si>
+    <t>**-*09-95-07</t>
+  </si>
+  <si>
+    <t>**-*09-61-05</t>
+  </si>
+  <si>
+    <t>**-*74-79-79</t>
+  </si>
+  <si>
+    <t>**-*73-73-15</t>
+  </si>
+  <si>
+    <t>**-*56-62-10</t>
+  </si>
+  <si>
+    <t>**-*50-56-42</t>
+  </si>
+  <si>
+    <t>**-*17-17-11</t>
+  </si>
+  <si>
+    <t>**-*98-01-70</t>
+  </si>
+  <si>
+    <t>**-*80-75-95</t>
+  </si>
+  <si>
+    <t>**-*67-01-83</t>
+  </si>
+  <si>
+    <t>**-*71-04-98</t>
+  </si>
+  <si>
+    <t>**-*43-43-86</t>
+  </si>
+  <si>
+    <t>**-*56-27-85</t>
+  </si>
+  <si>
+    <t>**-*58-11-17</t>
+  </si>
+  <si>
+    <t>**-*70-84-21</t>
+  </si>
+  <si>
+    <t>**-*72-26-07</t>
+  </si>
+  <si>
+    <t>**-*12-76-20</t>
+  </si>
+  <si>
+    <t>**-*14-18-10</t>
+  </si>
+  <si>
+    <t>**-*38-98-00</t>
+  </si>
+  <si>
+    <t>**-*91-65-66</t>
+  </si>
+  <si>
+    <t>**-*08-01-02</t>
+  </si>
+  <si>
+    <t>**-*60-06-91</t>
+  </si>
+  <si>
+    <t>**-*78-58-77</t>
+  </si>
+  <si>
+    <t>**-*96-23-07</t>
+  </si>
+  <si>
+    <t>**-*08-84-72</t>
+  </si>
+  <si>
+    <t>**-*84-90-88</t>
+  </si>
+  <si>
+    <t>**-*86-67-72</t>
+  </si>
+  <si>
+    <t>**-*22-97-79</t>
+  </si>
+  <si>
+    <t>**-*93-94-98</t>
+  </si>
+  <si>
+    <t>**-*22-95-05</t>
+  </si>
+  <si>
+    <t>**-*33-11-14</t>
+  </si>
+  <si>
+    <t>**-*13-44-51</t>
+  </si>
+  <si>
+    <t>**-*76-25-28</t>
+  </si>
+  <si>
+    <t>**-*27-58-84</t>
+  </si>
+  <si>
+    <t>**-*48-08-60</t>
+  </si>
+  <si>
+    <t>**-*80-55-30</t>
+  </si>
+  <si>
+    <t>**-*76-35-81</t>
+  </si>
+  <si>
+    <t>**-*03-36-84</t>
+  </si>
+  <si>
+    <t>**-*24-76-72</t>
+  </si>
+  <si>
+    <t>**-*16-48-47</t>
+  </si>
+  <si>
+    <t>**-*00-13-74</t>
+  </si>
+  <si>
+    <t>**-*42-83-38</t>
+  </si>
+  <si>
+    <t>**-*42-19-54</t>
+  </si>
+  <si>
+    <t>**-*65-20-01</t>
+  </si>
+  <si>
+    <t>**-*00-88-65</t>
+  </si>
+  <si>
+    <t>**-*10-99-93</t>
+  </si>
+  <si>
+    <t>**-*63-47-57</t>
+  </si>
+  <si>
+    <t>**-*00-28-29</t>
+  </si>
+  <si>
+    <t>**-*07-69-71</t>
+  </si>
+  <si>
+    <t>**-*76-19-59</t>
+  </si>
+  <si>
+    <t>**-*28-25-98</t>
+  </si>
+  <si>
+    <t>**-*82-95-07</t>
+  </si>
+  <si>
+    <t>**-*78-06-77</t>
+  </si>
+  <si>
+    <t>**-*01-93-00</t>
+  </si>
+  <si>
+    <t>**-*52-88-65</t>
+  </si>
+  <si>
+    <t>**-*06-26-50</t>
+  </si>
+  <si>
+    <t>**-*25-25-36</t>
+  </si>
+  <si>
+    <t>**-*52-37-20</t>
+  </si>
+  <si>
+    <t>**-*95-21-60</t>
+  </si>
+  <si>
+    <t>**-*79-58-90</t>
+  </si>
+  <si>
+    <t>**-*71-21-92</t>
+  </si>
+  <si>
+    <t>**-*94-21-01</t>
+  </si>
+  <si>
+    <t>**-*43-11-76</t>
+  </si>
+  <si>
+    <t>**-*89-93-77</t>
+  </si>
+  <si>
+    <t>**-*12-04-94</t>
+  </si>
+  <si>
+    <t>**-*42-46-81</t>
+  </si>
+  <si>
+    <t>**-*03-88-37</t>
+  </si>
+  <si>
+    <t>**-*56-57-75</t>
+  </si>
+  <si>
+    <t>**-*73-24-88</t>
+  </si>
+  <si>
+    <t>**-*64-77-81</t>
+  </si>
+  <si>
+    <t>**-*93-88-31</t>
+  </si>
+  <si>
+    <t>**-*38-42-82</t>
+  </si>
+  <si>
+    <t>**-*94-31-31</t>
+  </si>
+  <si>
+    <t>**-*78-00-68</t>
+  </si>
+  <si>
+    <t>**-*61-72-09</t>
+  </si>
+  <si>
+    <t>**-*32-36-41</t>
+  </si>
+  <si>
+    <t>**-*88-41-93</t>
+  </si>
+  <si>
+    <t>**-*06-38-39</t>
+  </si>
+  <si>
+    <t>**-*00-68-98</t>
+  </si>
+  <si>
+    <t>**-*11-40-37</t>
+  </si>
+  <si>
+    <t>**-*12-89-69</t>
+  </si>
+  <si>
+    <t>**-*69-55-60</t>
+  </si>
+  <si>
+    <t>**-*44-06-33</t>
+  </si>
+  <si>
+    <t>**-*70-08-33</t>
+  </si>
+  <si>
+    <t>**-*59-91-99</t>
+  </si>
+  <si>
+    <t>**-*47-97-00</t>
+  </si>
+  <si>
+    <t>**-*40-70-03</t>
+  </si>
+  <si>
+    <t>**-*93-47-77</t>
+  </si>
+  <si>
+    <t>**-*53-09-21</t>
+  </si>
+  <si>
+    <t>**-*14-05-16</t>
+  </si>
+  <si>
+    <t>**-*03-53-83</t>
+  </si>
+  <si>
+    <t>**-*66-94-91</t>
+  </si>
+  <si>
+    <t>**-*94-01-81</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="dd\-mm\-yyyy\ hh:mm:ss"/>
+    <numFmt numFmtId="171" formatCode="dd\-mm\-yyyy\ hh:mm"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -2984,7 +3591,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -3012,6 +3619,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -3328,14 +3938,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA66EC08-8D26-46AA-A6AA-1D6A0B4C73D5}">
-  <dimension ref="A7:C973"/>
+  <dimension ref="A7:H973"/>
   <sheetFormatPr defaultRowHeight="21" thickBottom="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="25.28515625" customWidth="1"/>
     <col min="3" max="3" width="26" style="5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.5703125" customWidth="1"/>
+    <col min="7" max="7" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="29.28515625" style="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="7" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3">
         <v>1</v>
       </c>
@@ -3345,8 +3958,17 @@
       <c r="C7" s="5">
         <v>46093.425000000003</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F7" s="3">
+        <v>1</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>951</v>
+      </c>
+      <c r="H7" s="10">
+        <v>46094.332638888889</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4">
         <v>2</v>
       </c>
@@ -3356,8 +3978,17 @@
       <c r="C8" s="5">
         <v>46093.421527777777</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F8" s="4">
+        <v>2</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>952</v>
+      </c>
+      <c r="H8" s="10">
+        <v>46094.331944444442</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4">
         <v>3</v>
       </c>
@@ -3367,8 +3998,17 @@
       <c r="C9" s="5">
         <v>46093.418749999997</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F9" s="4">
+        <v>3</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>953</v>
+      </c>
+      <c r="H9" s="10">
+        <v>46094.331944444442</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4">
         <v>4</v>
       </c>
@@ -3378,8 +4018,17 @@
       <c r="C10" s="5">
         <v>46093.415972222225</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F10" s="4">
+        <v>4</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>954</v>
+      </c>
+      <c r="H10" s="10">
+        <v>46094.322222222225</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4">
         <v>5</v>
       </c>
@@ -3389,8 +4038,17 @@
       <c r="C11" s="5">
         <v>46093.415277777778</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F11" s="4">
+        <v>5</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>955</v>
+      </c>
+      <c r="H11" s="10">
+        <v>46094.321527777778</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4">
         <v>6</v>
       </c>
@@ -3400,8 +4058,17 @@
       <c r="C12" s="5">
         <v>46093.414583333331</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F12" s="4">
+        <v>6</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>956</v>
+      </c>
+      <c r="H12" s="10">
+        <v>46094.320833333331</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="4">
         <v>7</v>
       </c>
@@ -3411,8 +4078,17 @@
       <c r="C13" s="5">
         <v>46093.414583333331</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F13" s="4">
+        <v>7</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>957</v>
+      </c>
+      <c r="H13" s="10">
+        <v>46094.320138888892</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="4">
         <v>8</v>
       </c>
@@ -3422,8 +4098,17 @@
       <c r="C14" s="5">
         <v>46093.413888888892</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F14" s="4">
+        <v>8</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>958</v>
+      </c>
+      <c r="H14" s="10">
+        <v>46094.308333333334</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="4">
         <v>9</v>
       </c>
@@ -3433,8 +4118,17 @@
       <c r="C15" s="5">
         <v>46093.413888888892</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F15" s="4">
+        <v>9</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>959</v>
+      </c>
+      <c r="H15" s="10">
+        <v>46094.306944444441</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="4">
         <v>10</v>
       </c>
@@ -3444,8 +4138,17 @@
       <c r="C16" s="5">
         <v>46093.411805555559</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F16" s="4">
+        <v>10</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>960</v>
+      </c>
+      <c r="H16" s="10">
+        <v>46094.298611111109</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="4">
         <v>11</v>
       </c>
@@ -3455,8 +4158,17 @@
       <c r="C17" s="5">
         <v>46093.411111111112</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F17" s="4">
+        <v>11</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>961</v>
+      </c>
+      <c r="H17" s="10">
+        <v>46094.290277777778</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4">
         <v>12</v>
       </c>
@@ -3466,8 +4178,17 @@
       <c r="C18" s="5">
         <v>46093.411111111112</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F18" s="4">
+        <v>12</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>962</v>
+      </c>
+      <c r="H18" s="10">
+        <v>46094.284722222219</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="3">
         <v>13</v>
       </c>
@@ -3477,8 +4198,17 @@
       <c r="C19" s="5">
         <v>46093.409722222219</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F19" s="3">
+        <v>13</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>963</v>
+      </c>
+      <c r="H19" s="10">
+        <v>46094.272916666669</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="4">
         <v>14</v>
       </c>
@@ -3488,8 +4218,17 @@
       <c r="C20" s="5">
         <v>46093.40902777778</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F20" s="4">
+        <v>14</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>964</v>
+      </c>
+      <c r="H20" s="10">
+        <v>46094.267361111109</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="4">
         <v>15</v>
       </c>
@@ -3499,8 +4238,17 @@
       <c r="C21" s="5">
         <v>46093.40902777778</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F21" s="4">
+        <v>15</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>965</v>
+      </c>
+      <c r="H21" s="10">
+        <v>46094.265972222223</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="4">
         <v>16</v>
       </c>
@@ -3510,8 +4258,17 @@
       <c r="C22" s="5">
         <v>46093.408333333333</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F22" s="4">
+        <v>16</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>966</v>
+      </c>
+      <c r="H22" s="10">
+        <v>46094.255555555559</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="4">
         <v>17</v>
       </c>
@@ -3521,8 +4278,17 @@
       <c r="C23" s="5">
         <v>46093.406944444447</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F23" s="4">
+        <v>17</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>967</v>
+      </c>
+      <c r="H23" s="10">
+        <v>46094.238888888889</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="4">
         <v>18</v>
       </c>
@@ -3532,8 +4298,17 @@
       <c r="C24" s="5">
         <v>46093.406944444447</v>
       </c>
-    </row>
-    <row r="25" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F24" s="4">
+        <v>18</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>968</v>
+      </c>
+      <c r="H24" s="10">
+        <v>46094.231249999997</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="3">
         <v>1</v>
       </c>
@@ -3543,8 +4318,17 @@
       <c r="C25" s="5">
         <v>46093.40347222222</v>
       </c>
-    </row>
-    <row r="26" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F25" s="4">
+        <v>19</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>969</v>
+      </c>
+      <c r="H25" s="10">
+        <v>46094.224999999999</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="4">
         <v>2</v>
       </c>
@@ -3554,8 +4338,17 @@
       <c r="C26" s="5">
         <v>46093.402083333334</v>
       </c>
-    </row>
-    <row r="27" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F26" s="4">
+        <v>20</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>970</v>
+      </c>
+      <c r="H26" s="10">
+        <v>46094.220138888886</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="4">
         <v>3</v>
       </c>
@@ -3565,8 +4358,17 @@
       <c r="C27" s="5">
         <v>46093.401388888888</v>
       </c>
-    </row>
-    <row r="28" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F27" s="4">
+        <v>21</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>971</v>
+      </c>
+      <c r="H27" s="10">
+        <v>46094.216666666667</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="4">
         <v>4</v>
       </c>
@@ -3576,8 +4378,17 @@
       <c r="C28" s="5">
         <v>46093.401388888888</v>
       </c>
-    </row>
-    <row r="29" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F28" s="4">
+        <v>22</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>972</v>
+      </c>
+      <c r="H28" s="10">
+        <v>46094.198611111111</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="4">
         <v>5</v>
       </c>
@@ -3587,8 +4398,17 @@
       <c r="C29" s="5">
         <v>46093.400694444441</v>
       </c>
-    </row>
-    <row r="30" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F29" s="4">
+        <v>23</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>973</v>
+      </c>
+      <c r="H29" s="10">
+        <v>46094.197916666664</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="4">
         <v>6</v>
       </c>
@@ -3598,8 +4418,17 @@
       <c r="C30" s="5">
         <v>46093.4</v>
       </c>
-    </row>
-    <row r="31" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F30" s="4">
+        <v>24</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>974</v>
+      </c>
+      <c r="H30" s="10">
+        <v>46094.1875</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="4">
         <v>7</v>
       </c>
@@ -3609,8 +4438,17 @@
       <c r="C31" s="5">
         <v>46093.399305555555</v>
       </c>
-    </row>
-    <row r="32" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F31" s="3">
+        <v>25</v>
+      </c>
+      <c r="G31" s="1" t="s">
+        <v>975</v>
+      </c>
+      <c r="H31" s="10">
+        <v>46094.168055555558</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="4">
         <v>8</v>
       </c>
@@ -3620,8 +4458,17 @@
       <c r="C32" s="5">
         <v>46093.398611111108</v>
       </c>
-    </row>
-    <row r="33" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F32" s="4">
+        <v>26</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>976</v>
+      </c>
+      <c r="H32" s="10">
+        <v>46094.163194444445</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="4">
         <v>9</v>
       </c>
@@ -3631,8 +4478,17 @@
       <c r="C33" s="5">
         <v>46093.395138888889</v>
       </c>
-    </row>
-    <row r="34" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F33" s="4">
+        <v>27</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>977</v>
+      </c>
+      <c r="H33" s="10">
+        <v>46094.150694444441</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="4">
         <v>10</v>
       </c>
@@ -3642,8 +4498,17 @@
       <c r="C34" s="5">
         <v>46093.395138888889</v>
       </c>
-    </row>
-    <row r="35" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F34" s="4">
+        <v>28</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>978</v>
+      </c>
+      <c r="H34" s="10">
+        <v>46094.15</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="4">
         <v>11</v>
       </c>
@@ -3653,8 +4518,17 @@
       <c r="C35" s="5">
         <v>46093.394444444442</v>
       </c>
-    </row>
-    <row r="36" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F35" s="4">
+        <v>29</v>
+      </c>
+      <c r="G35" s="2" t="s">
+        <v>979</v>
+      </c>
+      <c r="H35" s="10">
+        <v>46094.15</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="4">
         <v>12</v>
       </c>
@@ -3664,8 +4538,17 @@
       <c r="C36" s="5">
         <v>46093.394444444442</v>
       </c>
-    </row>
-    <row r="37" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F36" s="4">
+        <v>30</v>
+      </c>
+      <c r="G36" s="2" t="s">
+        <v>980</v>
+      </c>
+      <c r="H36" s="10">
+        <v>46094.134027777778</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="3">
         <v>13</v>
       </c>
@@ -3675,8 +4558,17 @@
       <c r="C37" s="5">
         <v>46093.388194444444</v>
       </c>
-    </row>
-    <row r="38" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F37" s="4">
+        <v>31</v>
+      </c>
+      <c r="G37" s="2" t="s">
+        <v>981</v>
+      </c>
+      <c r="H37" s="10">
+        <v>46094.132638888892</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="4">
         <v>14</v>
       </c>
@@ -3686,8 +4578,17 @@
       <c r="C38" s="5">
         <v>46093.388194444444</v>
       </c>
-    </row>
-    <row r="39" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F38" s="4">
+        <v>32</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>982</v>
+      </c>
+      <c r="H38" s="10">
+        <v>46094.109027777777</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="4">
         <v>15</v>
       </c>
@@ -3697,8 +4598,17 @@
       <c r="C39" s="5">
         <v>46093.385416666664</v>
       </c>
-    </row>
-    <row r="40" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F39" s="4">
+        <v>33</v>
+      </c>
+      <c r="G39" s="2" t="s">
+        <v>983</v>
+      </c>
+      <c r="H39" s="10">
+        <v>46094.081944444442</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="4">
         <v>16</v>
       </c>
@@ -3708,8 +4618,17 @@
       <c r="C40" s="5">
         <v>46093.384027777778</v>
       </c>
-    </row>
-    <row r="41" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F40" s="4">
+        <v>34</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>984</v>
+      </c>
+      <c r="H40" s="10">
+        <v>46094.081250000003</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="4">
         <v>17</v>
       </c>
@@ -3719,8 +4638,17 @@
       <c r="C41" s="5">
         <v>46093.383333333331</v>
       </c>
-    </row>
-    <row r="42" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F41" s="4">
+        <v>35</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>985</v>
+      </c>
+      <c r="H41" s="10">
+        <v>46094.071527777778</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="4">
         <v>18</v>
       </c>
@@ -3730,8 +4658,17 @@
       <c r="C42" s="5">
         <v>46093.381249999999</v>
       </c>
-    </row>
-    <row r="43" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F42" s="4">
+        <v>36</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>986</v>
+      </c>
+      <c r="H42" s="10">
+        <v>46094.038194444445</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="4">
         <v>19</v>
       </c>
@@ -3741,8 +4678,17 @@
       <c r="C43" s="5">
         <v>46093.377083333333</v>
       </c>
-    </row>
-    <row r="44" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F43" s="3">
+        <v>37</v>
+      </c>
+      <c r="G43" s="1" t="s">
+        <v>987</v>
+      </c>
+      <c r="H43" s="10">
+        <v>46094.003472222219</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="4">
         <v>20</v>
       </c>
@@ -3752,8 +4698,17 @@
       <c r="C44" s="5">
         <v>46093.370833333334</v>
       </c>
-    </row>
-    <row r="45" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F44" s="4">
+        <v>38</v>
+      </c>
+      <c r="G44" s="2" t="s">
+        <v>988</v>
+      </c>
+      <c r="H44" s="10">
+        <v>46093.994444444441</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="4">
         <v>21</v>
       </c>
@@ -3763,8 +4718,17 @@
       <c r="C45" s="5">
         <v>46093.351388888892</v>
       </c>
-    </row>
-    <row r="46" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F45" s="4">
+        <v>39</v>
+      </c>
+      <c r="G45" s="2" t="s">
+        <v>989</v>
+      </c>
+      <c r="H45" s="10">
+        <v>46093.988194444442</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="4">
         <v>22</v>
       </c>
@@ -3774,8 +4738,17 @@
       <c r="C46" s="5">
         <v>46093.336805555555</v>
       </c>
-    </row>
-    <row r="47" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F46" s="4">
+        <v>40</v>
+      </c>
+      <c r="G46" s="2" t="s">
+        <v>990</v>
+      </c>
+      <c r="H46" s="10">
+        <v>46093.98541666667</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="4">
         <v>23</v>
       </c>
@@ -3785,8 +4758,17 @@
       <c r="C47" s="5">
         <v>46093.306944444441</v>
       </c>
-    </row>
-    <row r="48" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F47" s="4">
+        <v>41</v>
+      </c>
+      <c r="G47" s="2" t="s">
+        <v>991</v>
+      </c>
+      <c r="H47" s="10">
+        <v>46093.984027777777</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="4">
         <v>24</v>
       </c>
@@ -3796,8 +4778,17 @@
       <c r="C48" s="5">
         <v>46093.296527777777</v>
       </c>
-    </row>
-    <row r="49" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F48" s="4">
+        <v>42</v>
+      </c>
+      <c r="G48" s="2" t="s">
+        <v>992</v>
+      </c>
+      <c r="H48" s="10">
+        <v>46093.976388888892</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A49" s="3">
         <v>25</v>
       </c>
@@ -3807,8 +4798,17 @@
       <c r="C49" s="5">
         <v>46093.306944444441</v>
       </c>
-    </row>
-    <row r="50" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F49" s="4">
+        <v>43</v>
+      </c>
+      <c r="G49" s="2" t="s">
+        <v>993</v>
+      </c>
+      <c r="H49" s="10">
+        <v>46093.973611111112</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="4">
         <v>26</v>
       </c>
@@ -3818,8 +4818,17 @@
       <c r="C50" s="5">
         <v>46093.296527777777</v>
       </c>
-    </row>
-    <row r="51" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F50" s="4">
+        <v>44</v>
+      </c>
+      <c r="G50" s="2" t="s">
+        <v>994</v>
+      </c>
+      <c r="H50" s="10">
+        <v>46093.972916666666</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="4">
         <v>27</v>
       </c>
@@ -3829,8 +4838,17 @@
       <c r="C51" s="5">
         <v>46093.236805555556</v>
       </c>
-    </row>
-    <row r="52" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F51" s="4">
+        <v>45</v>
+      </c>
+      <c r="G51" s="2" t="s">
+        <v>995</v>
+      </c>
+      <c r="H51" s="10">
+        <v>46093.961805555555</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="4">
         <v>28</v>
       </c>
@@ -3840,8 +4858,17 @@
       <c r="C52" s="5">
         <v>46092.972916666666</v>
       </c>
-    </row>
-    <row r="53" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F52" s="4">
+        <v>46</v>
+      </c>
+      <c r="G52" s="2" t="s">
+        <v>996</v>
+      </c>
+      <c r="H52" s="10">
+        <v>46093.961111111108</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="4">
         <v>29</v>
       </c>
@@ -3851,8 +4878,17 @@
       <c r="C53" s="5">
         <v>46092.944444444445</v>
       </c>
-    </row>
-    <row r="54" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F53" s="4">
+        <v>47</v>
+      </c>
+      <c r="G53" s="2" t="s">
+        <v>997</v>
+      </c>
+      <c r="H53" s="10">
+        <v>46093.959722222222</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="4">
         <v>30</v>
       </c>
@@ -3862,8 +4898,17 @@
       <c r="C54" s="5">
         <v>46092.943055555559</v>
       </c>
-    </row>
-    <row r="55" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F54" s="4">
+        <v>48</v>
+      </c>
+      <c r="G54" s="2" t="s">
+        <v>998</v>
+      </c>
+      <c r="H54" s="10">
+        <v>46093.957638888889</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A55" s="4">
         <v>31</v>
       </c>
@@ -3873,8 +4918,17 @@
       <c r="C55" s="5">
         <v>46092.9375</v>
       </c>
-    </row>
-    <row r="56" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F55" s="3">
+        <v>49</v>
+      </c>
+      <c r="G55" s="1" t="s">
+        <v>999</v>
+      </c>
+      <c r="H55" s="10">
+        <v>46093.956250000003</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A56" s="4">
         <v>32</v>
       </c>
@@ -3884,8 +4938,17 @@
       <c r="C56" s="5">
         <v>46092.934027777781</v>
       </c>
-    </row>
-    <row r="57" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F56" s="4">
+        <v>50</v>
+      </c>
+      <c r="G56" s="2" t="s">
+        <v>1000</v>
+      </c>
+      <c r="H56" s="10">
+        <v>46093.954861111109</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A57" s="4">
         <v>33</v>
       </c>
@@ -3895,8 +4958,17 @@
       <c r="C57" s="5">
         <v>46092.928472222222</v>
       </c>
-    </row>
-    <row r="58" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F57" s="4">
+        <v>51</v>
+      </c>
+      <c r="G57" s="2" t="s">
+        <v>1001</v>
+      </c>
+      <c r="H57" s="10">
+        <v>46093.950694444444</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A58" s="4">
         <v>34</v>
       </c>
@@ -3906,8 +4978,17 @@
       <c r="C58" s="5">
         <v>46092.927083333336</v>
       </c>
-    </row>
-    <row r="59" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F58" s="4">
+        <v>52</v>
+      </c>
+      <c r="G58" s="2" t="s">
+        <v>1002</v>
+      </c>
+      <c r="H58" s="10">
+        <v>46093.949305555558</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="4">
         <v>35</v>
       </c>
@@ -3917,8 +4998,17 @@
       <c r="C59" s="5">
         <v>46092.925000000003</v>
       </c>
-    </row>
-    <row r="60" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F59" s="4">
+        <v>53</v>
+      </c>
+      <c r="G59" s="2" t="s">
+        <v>1003</v>
+      </c>
+      <c r="H59" s="10">
+        <v>46093.945833333331</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A60" s="4">
         <v>36</v>
       </c>
@@ -3928,8 +5018,17 @@
       <c r="C60" s="5">
         <v>46092.924305555556</v>
       </c>
-    </row>
-    <row r="61" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F60" s="4">
+        <v>54</v>
+      </c>
+      <c r="G60" s="2" t="s">
+        <v>1004</v>
+      </c>
+      <c r="H60" s="10">
+        <v>46093.938888888886</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A61" s="3">
         <v>37</v>
       </c>
@@ -3939,8 +5038,17 @@
       <c r="C61" s="5">
         <v>46092.923611111109</v>
       </c>
-    </row>
-    <row r="62" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F61" s="4">
+        <v>55</v>
+      </c>
+      <c r="G61" s="2" t="s">
+        <v>1005</v>
+      </c>
+      <c r="H61" s="10">
+        <v>46093.921527777777</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A62" s="4">
         <v>38</v>
       </c>
@@ -3950,8 +5058,17 @@
       <c r="C62" s="5">
         <v>46092.921527777777</v>
       </c>
-    </row>
-    <row r="63" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F62" s="4">
+        <v>56</v>
+      </c>
+      <c r="G62" s="2" t="s">
+        <v>1006</v>
+      </c>
+      <c r="H62" s="10">
+        <v>46093.92083333333</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A63" s="4">
         <v>39</v>
       </c>
@@ -3961,8 +5078,17 @@
       <c r="C63" s="5">
         <v>46092.921527777777</v>
       </c>
-    </row>
-    <row r="64" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F63" s="4">
+        <v>57</v>
+      </c>
+      <c r="G63" s="2" t="s">
+        <v>1007</v>
+      </c>
+      <c r="H63" s="10">
+        <v>46093.920138888891</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A64" s="4">
         <v>40</v>
       </c>
@@ -3972,8 +5098,17 @@
       <c r="C64" s="5">
         <v>46092.919444444444</v>
       </c>
-    </row>
-    <row r="65" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F64" s="4">
+        <v>58</v>
+      </c>
+      <c r="G64" s="2" t="s">
+        <v>1008</v>
+      </c>
+      <c r="H64" s="10">
+        <v>46093.919444444444</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A65" s="4">
         <v>41</v>
       </c>
@@ -3983,8 +5118,17 @@
       <c r="C65" s="5">
         <v>46092.918055555558</v>
       </c>
-    </row>
-    <row r="66" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F65" s="4">
+        <v>59</v>
+      </c>
+      <c r="G65" s="2" t="s">
+        <v>1009</v>
+      </c>
+      <c r="H65" s="10">
+        <v>46093.915972222225</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="4">
         <v>42</v>
       </c>
@@ -3994,8 +5138,17 @@
       <c r="C66" s="5">
         <v>46092.916666666664</v>
       </c>
-    </row>
-    <row r="67" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F66" s="4">
+        <v>60</v>
+      </c>
+      <c r="G66" s="2" t="s">
+        <v>1010</v>
+      </c>
+      <c r="H66" s="10">
+        <v>46093.912499999999</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A67" s="4">
         <v>43</v>
       </c>
@@ -4005,8 +5158,17 @@
       <c r="C67" s="5">
         <v>46092.915972222225</v>
       </c>
-    </row>
-    <row r="68" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F67" s="3">
+        <v>61</v>
+      </c>
+      <c r="G67" s="1" t="s">
+        <v>1011</v>
+      </c>
+      <c r="H67" s="10">
+        <v>46093.910416666666</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A68" s="4">
         <v>44</v>
       </c>
@@ -4016,8 +5178,17 @@
       <c r="C68" s="5">
         <v>46092.910416666666</v>
       </c>
-    </row>
-    <row r="69" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F68" s="4">
+        <v>62</v>
+      </c>
+      <c r="G68" s="2" t="s">
+        <v>1012</v>
+      </c>
+      <c r="H68" s="10">
+        <v>46093.90902777778</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A69" s="4">
         <v>45</v>
       </c>
@@ -4027,8 +5198,17 @@
       <c r="C69" s="5">
         <v>46092.909722222219</v>
       </c>
-    </row>
-    <row r="70" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F69" s="4">
+        <v>63</v>
+      </c>
+      <c r="G69" s="2" t="s">
+        <v>1013</v>
+      </c>
+      <c r="H69" s="10">
+        <v>46093.90625</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A70" s="4">
         <v>46</v>
       </c>
@@ -4038,8 +5218,17 @@
       <c r="C70" s="5">
         <v>46092.90902777778</v>
       </c>
-    </row>
-    <row r="71" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F70" s="4">
+        <v>64</v>
+      </c>
+      <c r="G70" s="2" t="s">
+        <v>1014</v>
+      </c>
+      <c r="H70" s="10">
+        <v>46093.90625</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A71" s="4">
         <v>47</v>
       </c>
@@ -4049,8 +5238,17 @@
       <c r="C71" s="5">
         <v>46092.907638888886</v>
       </c>
-    </row>
-    <row r="72" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F71" s="4">
+        <v>65</v>
+      </c>
+      <c r="G71" s="2" t="s">
+        <v>1015</v>
+      </c>
+      <c r="H71" s="10">
+        <v>46093.899305555555</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A72" s="4">
         <v>48</v>
       </c>
@@ -4060,8 +5258,17 @@
       <c r="C72" s="5">
         <v>46092.905555555553</v>
       </c>
-    </row>
-    <row r="73" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F72" s="4">
+        <v>66</v>
+      </c>
+      <c r="G72" s="2" t="s">
+        <v>1016</v>
+      </c>
+      <c r="H72" s="10">
+        <v>46093.897222222222</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A73" s="3">
         <v>49</v>
       </c>
@@ -4071,8 +5278,17 @@
       <c r="C73" s="5">
         <v>46092.904861111114</v>
       </c>
-    </row>
-    <row r="74" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F73" s="4">
+        <v>67</v>
+      </c>
+      <c r="G73" s="2" t="s">
+        <v>1017</v>
+      </c>
+      <c r="H73" s="10">
+        <v>46093.897222222222</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A74" s="4">
         <v>50</v>
       </c>
@@ -4082,8 +5298,17 @@
       <c r="C74" s="5">
         <v>46092.902777777781</v>
       </c>
-    </row>
-    <row r="75" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F74" s="4">
+        <v>68</v>
+      </c>
+      <c r="G74" s="2" t="s">
+        <v>1018</v>
+      </c>
+      <c r="H74" s="10">
+        <v>46093.895138888889</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A75" s="4">
         <v>51</v>
       </c>
@@ -4093,8 +5318,17 @@
       <c r="C75" s="5">
         <v>46092.901388888888</v>
       </c>
-    </row>
-    <row r="76" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F75" s="4">
+        <v>69</v>
+      </c>
+      <c r="G75" s="2" t="s">
+        <v>1019</v>
+      </c>
+      <c r="H75" s="10">
+        <v>46093.893750000003</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A76" s="4">
         <v>52</v>
       </c>
@@ -4104,8 +5338,17 @@
       <c r="C76" s="5">
         <v>46092.897222222222</v>
       </c>
-    </row>
-    <row r="77" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F76" s="4">
+        <v>70</v>
+      </c>
+      <c r="G76" s="2" t="s">
+        <v>1020</v>
+      </c>
+      <c r="H76" s="10">
+        <v>46093.892361111109</v>
+      </c>
+    </row>
+    <row r="77" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A77" s="4">
         <v>53</v>
       </c>
@@ -4115,8 +5358,17 @@
       <c r="C77" s="5">
         <v>46092.893750000003</v>
       </c>
-    </row>
-    <row r="78" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F77" s="4">
+        <v>71</v>
+      </c>
+      <c r="G77" s="2" t="s">
+        <v>1021</v>
+      </c>
+      <c r="H77" s="10">
+        <v>46093.89166666667</v>
+      </c>
+    </row>
+    <row r="78" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A78" s="4">
         <v>54</v>
       </c>
@@ -4126,8 +5378,17 @@
       <c r="C78" s="5">
         <v>46092.892361111109</v>
       </c>
-    </row>
-    <row r="79" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F78" s="4">
+        <v>72</v>
+      </c>
+      <c r="G78" s="2" t="s">
+        <v>1022</v>
+      </c>
+      <c r="H78" s="10">
+        <v>46093.890972222223</v>
+      </c>
+    </row>
+    <row r="79" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A79" s="4">
         <v>55</v>
       </c>
@@ -4137,8 +5398,17 @@
       <c r="C79" s="5">
         <v>46092.890972222223</v>
       </c>
-    </row>
-    <row r="80" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F79" s="3">
+        <v>73</v>
+      </c>
+      <c r="G79" s="1" t="s">
+        <v>1023</v>
+      </c>
+      <c r="H79" s="10">
+        <v>46093.890972222223</v>
+      </c>
+    </row>
+    <row r="80" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A80" s="4">
         <v>56</v>
       </c>
@@ -4148,8 +5418,17 @@
       <c r="C80" s="5">
         <v>46092.890972222223</v>
       </c>
-    </row>
-    <row r="81" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F80" s="4">
+        <v>74</v>
+      </c>
+      <c r="G80" s="2" t="s">
+        <v>1024</v>
+      </c>
+      <c r="H80" s="10">
+        <v>46093.890277777777</v>
+      </c>
+    </row>
+    <row r="81" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A81" s="4">
         <v>57</v>
       </c>
@@ -4159,8 +5438,17 @@
       <c r="C81" s="5">
         <v>46092.890277777777</v>
       </c>
-    </row>
-    <row r="82" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F81" s="4">
+        <v>75</v>
+      </c>
+      <c r="G81" s="2" t="s">
+        <v>1025</v>
+      </c>
+      <c r="H81" s="10">
+        <v>46093.888194444444</v>
+      </c>
+    </row>
+    <row r="82" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A82" s="4">
         <v>58</v>
       </c>
@@ -4170,8 +5458,17 @@
       <c r="C82" s="5">
         <v>46092.888194444444</v>
       </c>
-    </row>
-    <row r="83" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F82" s="4">
+        <v>76</v>
+      </c>
+      <c r="G82" s="2" t="s">
+        <v>1026</v>
+      </c>
+      <c r="H82" s="10">
+        <v>46093.886111111111</v>
+      </c>
+    </row>
+    <row r="83" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A83" s="4">
         <v>59</v>
       </c>
@@ -4181,8 +5478,17 @@
       <c r="C83" s="5">
         <v>46092.888194444444</v>
       </c>
-    </row>
-    <row r="84" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F83" s="4">
+        <v>77</v>
+      </c>
+      <c r="G83" s="2" t="s">
+        <v>1027</v>
+      </c>
+      <c r="H83" s="10">
+        <v>46093.884722222225</v>
+      </c>
+    </row>
+    <row r="84" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A84" s="4">
         <v>60</v>
       </c>
@@ -4192,8 +5498,17 @@
       <c r="C84" s="5">
         <v>46092.886111111111</v>
       </c>
-    </row>
-    <row r="85" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F84" s="4">
+        <v>78</v>
+      </c>
+      <c r="G84" s="2" t="s">
+        <v>1028</v>
+      </c>
+      <c r="H84" s="10">
+        <v>46093.884722222225</v>
+      </c>
+    </row>
+    <row r="85" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A85" s="3">
         <v>61</v>
       </c>
@@ -4203,8 +5518,17 @@
       <c r="C85" s="5">
         <v>46092.886111111111</v>
       </c>
-    </row>
-    <row r="86" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F85" s="4">
+        <v>79</v>
+      </c>
+      <c r="G85" s="2" t="s">
+        <v>1029</v>
+      </c>
+      <c r="H85" s="10">
+        <v>46093.883333333331</v>
+      </c>
+    </row>
+    <row r="86" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A86" s="4">
         <v>62</v>
       </c>
@@ -4214,8 +5538,17 @@
       <c r="C86" s="5">
         <v>46092.884027777778</v>
       </c>
-    </row>
-    <row r="87" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F86" s="4">
+        <v>80</v>
+      </c>
+      <c r="G86" s="2" t="s">
+        <v>1030</v>
+      </c>
+      <c r="H86" s="10">
+        <v>46093.881944444445</v>
+      </c>
+    </row>
+    <row r="87" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A87" s="4">
         <v>63</v>
       </c>
@@ -4225,8 +5558,17 @@
       <c r="C87" s="5">
         <v>46092.883333333331</v>
       </c>
-    </row>
-    <row r="88" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F87" s="4">
+        <v>81</v>
+      </c>
+      <c r="G87" s="2" t="s">
+        <v>1031</v>
+      </c>
+      <c r="H87" s="10">
+        <v>46093.881249999999</v>
+      </c>
+    </row>
+    <row r="88" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A88" s="4">
         <v>64</v>
       </c>
@@ -4236,8 +5578,17 @@
       <c r="C88" s="5">
         <v>46092.882638888892</v>
       </c>
-    </row>
-    <row r="89" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F88" s="4">
+        <v>82</v>
+      </c>
+      <c r="G88" s="2" t="s">
+        <v>1032</v>
+      </c>
+      <c r="H88" s="10">
+        <v>46093.880555555559</v>
+      </c>
+    </row>
+    <row r="89" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A89" s="4">
         <v>65</v>
       </c>
@@ -4247,8 +5598,17 @@
       <c r="C89" s="5">
         <v>46092.880555555559</v>
       </c>
-    </row>
-    <row r="90" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F89" s="4">
+        <v>83</v>
+      </c>
+      <c r="G89" s="2" t="s">
+        <v>1033</v>
+      </c>
+      <c r="H89" s="10">
+        <v>46093.878472222219</v>
+      </c>
+    </row>
+    <row r="90" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A90" s="4">
         <v>66</v>
       </c>
@@ -4258,8 +5618,17 @@
       <c r="C90" s="5">
         <v>46092.879861111112</v>
       </c>
-    </row>
-    <row r="91" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F90" s="4">
+        <v>84</v>
+      </c>
+      <c r="G90" s="2" t="s">
+        <v>1034</v>
+      </c>
+      <c r="H90" s="10">
+        <v>46093.87777777778</v>
+      </c>
+    </row>
+    <row r="91" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A91" s="4">
         <v>67</v>
       </c>
@@ -4269,8 +5638,17 @@
       <c r="C91" s="5">
         <v>46092.879861111112</v>
       </c>
-    </row>
-    <row r="92" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F91" s="3">
+        <v>85</v>
+      </c>
+      <c r="G91" s="1" t="s">
+        <v>1035</v>
+      </c>
+      <c r="H91" s="10">
+        <v>46093.877083333333</v>
+      </c>
+    </row>
+    <row r="92" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A92" s="4">
         <v>68</v>
       </c>
@@ -4280,8 +5658,17 @@
       <c r="C92" s="5">
         <v>46092.879166666666</v>
       </c>
-    </row>
-    <row r="93" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F92" s="4">
+        <v>86</v>
+      </c>
+      <c r="G92" s="2" t="s">
+        <v>1036</v>
+      </c>
+      <c r="H92" s="10">
+        <v>46093.873611111114</v>
+      </c>
+    </row>
+    <row r="93" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A93" s="4">
         <v>69</v>
       </c>
@@ -4291,8 +5678,17 @@
       <c r="C93" s="5">
         <v>46092.87777777778</v>
       </c>
-    </row>
-    <row r="94" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F93" s="4">
+        <v>87</v>
+      </c>
+      <c r="G93" s="2" t="s">
+        <v>1037</v>
+      </c>
+      <c r="H93" s="10">
+        <v>46093.872916666667</v>
+      </c>
+    </row>
+    <row r="94" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A94" s="4">
         <v>70</v>
       </c>
@@ -4302,8 +5698,17 @@
       <c r="C94" s="5">
         <v>46092.875</v>
       </c>
-    </row>
-    <row r="95" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F94" s="4">
+        <v>88</v>
+      </c>
+      <c r="G94" s="2" t="s">
+        <v>1038</v>
+      </c>
+      <c r="H94" s="10">
+        <v>46093.867361111108</v>
+      </c>
+    </row>
+    <row r="95" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A95" s="4">
         <v>71</v>
       </c>
@@ -4313,8 +5718,17 @@
       <c r="C95" s="5">
         <v>46092.874305555553</v>
       </c>
-    </row>
-    <row r="96" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F95" s="4">
+        <v>89</v>
+      </c>
+      <c r="G95" s="2" t="s">
+        <v>1039</v>
+      </c>
+      <c r="H95" s="10">
+        <v>46093.863888888889</v>
+      </c>
+    </row>
+    <row r="96" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A96" s="4">
         <v>72</v>
       </c>
@@ -4324,8 +5738,17 @@
       <c r="C96" s="5">
         <v>46092.872916666667</v>
       </c>
-    </row>
-    <row r="97" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F96" s="4">
+        <v>90</v>
+      </c>
+      <c r="G96" s="2" t="s">
+        <v>1040</v>
+      </c>
+      <c r="H96" s="10">
+        <v>46093.859722222223</v>
+      </c>
+    </row>
+    <row r="97" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A97" s="3">
         <v>73</v>
       </c>
@@ -4335,8 +5758,17 @@
       <c r="C97" s="5">
         <v>46092.87222222222</v>
       </c>
-    </row>
-    <row r="98" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F97" s="4">
+        <v>91</v>
+      </c>
+      <c r="G97" s="2" t="s">
+        <v>1041</v>
+      </c>
+      <c r="H97" s="10">
+        <v>46093.855555555558</v>
+      </c>
+    </row>
+    <row r="98" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A98" s="4">
         <v>74</v>
       </c>
@@ -4346,8 +5778,17 @@
       <c r="C98" s="5">
         <v>46092.87222222222</v>
       </c>
-    </row>
-    <row r="99" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F98" s="4">
+        <v>92</v>
+      </c>
+      <c r="G98" s="2" t="s">
+        <v>1042</v>
+      </c>
+      <c r="H98" s="10">
+        <v>46093.852083333331</v>
+      </c>
+    </row>
+    <row r="99" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A99" s="4">
         <v>75</v>
       </c>
@@ -4357,8 +5798,17 @@
       <c r="C99" s="5">
         <v>46092.871527777781</v>
       </c>
-    </row>
-    <row r="100" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F99" s="4">
+        <v>93</v>
+      </c>
+      <c r="G99" s="2" t="s">
+        <v>1043</v>
+      </c>
+      <c r="H99" s="10">
+        <v>46093.828472222223</v>
+      </c>
+    </row>
+    <row r="100" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A100" s="4">
         <v>76</v>
       </c>
@@ -4368,8 +5818,17 @@
       <c r="C100" s="5">
         <v>46092.871527777781</v>
       </c>
-    </row>
-    <row r="101" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F100" s="4">
+        <v>94</v>
+      </c>
+      <c r="G100" s="2" t="s">
+        <v>1044</v>
+      </c>
+      <c r="H100" s="10">
+        <v>46093.826388888891</v>
+      </c>
+    </row>
+    <row r="101" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A101" s="4">
         <v>77</v>
       </c>
@@ -4379,8 +5838,17 @@
       <c r="C101" s="5">
         <v>46092.867361111108</v>
       </c>
-    </row>
-    <row r="102" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F101" s="4">
+        <v>95</v>
+      </c>
+      <c r="G101" s="2" t="s">
+        <v>1045</v>
+      </c>
+      <c r="H101" s="10">
+        <v>46093.824999999997</v>
+      </c>
+    </row>
+    <row r="102" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A102" s="4">
         <v>78</v>
       </c>
@@ -4390,8 +5858,17 @@
       <c r="C102" s="5">
         <v>46092.866666666669</v>
       </c>
-    </row>
-    <row r="103" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F102" s="4">
+        <v>96</v>
+      </c>
+      <c r="G102" s="2" t="s">
+        <v>1046</v>
+      </c>
+      <c r="H102" s="10">
+        <v>46093.818055555559</v>
+      </c>
+    </row>
+    <row r="103" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A103" s="4">
         <v>79</v>
       </c>
@@ -4401,8 +5878,17 @@
       <c r="C103" s="5">
         <v>46092.866666666669</v>
       </c>
-    </row>
-    <row r="104" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F103" s="3">
+        <v>97</v>
+      </c>
+      <c r="G103" s="1" t="s">
+        <v>1047</v>
+      </c>
+      <c r="H103" s="10">
+        <v>46093.814583333333</v>
+      </c>
+    </row>
+    <row r="104" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A104" s="4">
         <v>80</v>
       </c>
@@ -4412,8 +5898,17 @@
       <c r="C104" s="5">
         <v>46092.862500000003</v>
       </c>
-    </row>
-    <row r="105" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F104" s="4">
+        <v>98</v>
+      </c>
+      <c r="G104" s="2" t="s">
+        <v>1048</v>
+      </c>
+      <c r="H104" s="10">
+        <v>46093.8</v>
+      </c>
+    </row>
+    <row r="105" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A105" s="4">
         <v>81</v>
       </c>
@@ -4423,8 +5918,17 @@
       <c r="C105" s="5">
         <v>46092.861805555556</v>
       </c>
-    </row>
-    <row r="106" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F105" s="4">
+        <v>99</v>
+      </c>
+      <c r="G105" s="2" t="s">
+        <v>1049</v>
+      </c>
+      <c r="H105" s="10">
+        <v>46093.769444444442</v>
+      </c>
+    </row>
+    <row r="106" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A106" s="4">
         <v>82</v>
       </c>
@@ -4434,8 +5938,17 @@
       <c r="C106" s="5">
         <v>46092.861111111109</v>
       </c>
-    </row>
-    <row r="107" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F106" s="4">
+        <v>100</v>
+      </c>
+      <c r="G106" s="2" t="s">
+        <v>1050</v>
+      </c>
+      <c r="H106" s="10">
+        <v>46093.768055555556</v>
+      </c>
+    </row>
+    <row r="107" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A107" s="4">
         <v>83</v>
       </c>
@@ -4445,8 +5958,17 @@
       <c r="C107" s="5">
         <v>46092.859722222223</v>
       </c>
-    </row>
-    <row r="108" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F107" s="4">
+        <v>101</v>
+      </c>
+      <c r="G107" s="2" t="s">
+        <v>1051</v>
+      </c>
+      <c r="H107" s="10">
+        <v>46093.759722222225</v>
+      </c>
+    </row>
+    <row r="108" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A108" s="4">
         <v>84</v>
       </c>
@@ -4456,8 +5978,17 @@
       <c r="C108" s="5">
         <v>46092.859027777777</v>
       </c>
-    </row>
-    <row r="109" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F108" s="4">
+        <v>102</v>
+      </c>
+      <c r="G108" s="2" t="s">
+        <v>1052</v>
+      </c>
+      <c r="H108" s="10">
+        <v>46093.758333333331</v>
+      </c>
+    </row>
+    <row r="109" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A109" s="3">
         <v>85</v>
       </c>
@@ -4467,8 +5998,17 @@
       <c r="C109" s="5">
         <v>46092.85833333333</v>
       </c>
-    </row>
-    <row r="110" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F109" s="4">
+        <v>103</v>
+      </c>
+      <c r="G109" s="2" t="s">
+        <v>1053</v>
+      </c>
+      <c r="H109" s="10">
+        <v>46093.754166666666</v>
+      </c>
+    </row>
+    <row r="110" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A110" s="4">
         <v>86</v>
       </c>
@@ -4478,8 +6018,17 @@
       <c r="C110" s="5">
         <v>46092.857638888891</v>
       </c>
-    </row>
-    <row r="111" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F110" s="4">
+        <v>104</v>
+      </c>
+      <c r="G110" s="2" t="s">
+        <v>1054</v>
+      </c>
+      <c r="H110" s="10">
+        <v>46093.75</v>
+      </c>
+    </row>
+    <row r="111" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A111" s="4">
         <v>87</v>
       </c>
@@ -4489,8 +6038,17 @@
       <c r="C111" s="5">
         <v>46092.856944444444</v>
       </c>
-    </row>
-    <row r="112" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F111" s="4">
+        <v>105</v>
+      </c>
+      <c r="G111" s="2" t="s">
+        <v>1055</v>
+      </c>
+      <c r="H111" s="10">
+        <v>46093.744444444441</v>
+      </c>
+    </row>
+    <row r="112" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A112" s="4">
         <v>88</v>
       </c>
@@ -4500,8 +6058,17 @@
       <c r="C112" s="5">
         <v>46092.856944444444</v>
       </c>
-    </row>
-    <row r="113" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F112" s="4">
+        <v>106</v>
+      </c>
+      <c r="G112" s="2" t="s">
+        <v>1056</v>
+      </c>
+      <c r="H112" s="10">
+        <v>46093.742361111108</v>
+      </c>
+    </row>
+    <row r="113" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A113" s="4">
         <v>89</v>
       </c>
@@ -4511,8 +6078,17 @@
       <c r="C113" s="5">
         <v>46092.854166666664</v>
       </c>
-    </row>
-    <row r="114" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F113" s="4">
+        <v>107</v>
+      </c>
+      <c r="G113" s="2" t="s">
+        <v>1057</v>
+      </c>
+      <c r="H113" s="10">
+        <v>46093.740972222222</v>
+      </c>
+    </row>
+    <row r="114" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A114" s="4">
         <v>90</v>
       </c>
@@ -4522,8 +6098,17 @@
       <c r="C114" s="5">
         <v>46092.853472222225</v>
       </c>
-    </row>
-    <row r="115" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F114" s="4">
+        <v>108</v>
+      </c>
+      <c r="G114" s="2" t="s">
+        <v>1058</v>
+      </c>
+      <c r="H114" s="10">
+        <v>46093.740277777775</v>
+      </c>
+    </row>
+    <row r="115" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A115" s="4">
         <v>91</v>
       </c>
@@ -4533,8 +6118,17 @@
       <c r="C115" s="5">
         <v>46092.852777777778</v>
       </c>
-    </row>
-    <row r="116" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F115" s="3">
+        <v>109</v>
+      </c>
+      <c r="G115" s="1" t="s">
+        <v>1059</v>
+      </c>
+      <c r="H115" s="10">
+        <v>46093.740277777775</v>
+      </c>
+    </row>
+    <row r="116" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A116" s="4">
         <v>92</v>
       </c>
@@ -4544,8 +6138,17 @@
       <c r="C116" s="5">
         <v>46092.851388888892</v>
       </c>
-    </row>
-    <row r="117" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F116" s="4">
+        <v>110</v>
+      </c>
+      <c r="G116" s="2" t="s">
+        <v>1060</v>
+      </c>
+      <c r="H116" s="10">
+        <v>46093.738888888889</v>
+      </c>
+    </row>
+    <row r="117" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A117" s="4">
         <v>93</v>
       </c>
@@ -4555,8 +6158,17 @@
       <c r="C117" s="5">
         <v>46092.851388888892</v>
       </c>
-    </row>
-    <row r="118" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F117" s="4">
+        <v>111</v>
+      </c>
+      <c r="G117" s="2" t="s">
+        <v>1061</v>
+      </c>
+      <c r="H117" s="10">
+        <v>46093.738888888889</v>
+      </c>
+    </row>
+    <row r="118" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A118" s="4">
         <v>94</v>
       </c>
@@ -4566,8 +6178,17 @@
       <c r="C118" s="5">
         <v>46092.849305555559</v>
       </c>
-    </row>
-    <row r="119" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F118" s="4">
+        <v>112</v>
+      </c>
+      <c r="G118" s="2" t="s">
+        <v>1062</v>
+      </c>
+      <c r="H118" s="10">
+        <v>46093.731944444444</v>
+      </c>
+    </row>
+    <row r="119" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A119" s="4">
         <v>95</v>
       </c>
@@ -4577,8 +6198,17 @@
       <c r="C119" s="5">
         <v>46092.84652777778</v>
       </c>
-    </row>
-    <row r="120" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F119" s="4">
+        <v>113</v>
+      </c>
+      <c r="G119" s="2" t="s">
+        <v>1063</v>
+      </c>
+      <c r="H119" s="10">
+        <v>46093.731944444444</v>
+      </c>
+    </row>
+    <row r="120" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A120" s="4">
         <v>96</v>
       </c>
@@ -4588,8 +6218,17 @@
       <c r="C120" s="5">
         <v>46092.845138888886</v>
       </c>
-    </row>
-    <row r="121" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F120" s="4">
+        <v>114</v>
+      </c>
+      <c r="G120" s="2" t="s">
+        <v>1064</v>
+      </c>
+      <c r="H120" s="10">
+        <v>46093.731249999997</v>
+      </c>
+    </row>
+    <row r="121" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A121" s="3">
         <v>97</v>
       </c>
@@ -4599,8 +6238,17 @@
       <c r="C121" s="5">
         <v>46092.842361111114</v>
       </c>
-    </row>
-    <row r="122" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F121" s="4">
+        <v>115</v>
+      </c>
+      <c r="G121" s="2" t="s">
+        <v>1065</v>
+      </c>
+      <c r="H121" s="10">
+        <v>46093.730555555558</v>
+      </c>
+    </row>
+    <row r="122" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A122" s="4">
         <v>98</v>
       </c>
@@ -4610,8 +6258,17 @@
       <c r="C122" s="5">
         <v>46092.841666666667</v>
       </c>
-    </row>
-    <row r="123" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F122" s="4">
+        <v>116</v>
+      </c>
+      <c r="G122" s="2" t="s">
+        <v>1066</v>
+      </c>
+      <c r="H122" s="10">
+        <v>46093.728472222225</v>
+      </c>
+    </row>
+    <row r="123" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A123" s="4">
         <v>99</v>
       </c>
@@ -4621,8 +6278,17 @@
       <c r="C123" s="5">
         <v>46092.838888888888</v>
       </c>
-    </row>
-    <row r="124" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F123" s="4">
+        <v>117</v>
+      </c>
+      <c r="G123" s="2" t="s">
+        <v>1067</v>
+      </c>
+      <c r="H123" s="10">
+        <v>46093.727777777778</v>
+      </c>
+    </row>
+    <row r="124" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A124" s="4">
         <v>100</v>
       </c>
@@ -4632,8 +6298,17 @@
       <c r="C124" s="5">
         <v>46092.838888888888</v>
       </c>
-    </row>
-    <row r="125" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F124" s="4">
+        <v>118</v>
+      </c>
+      <c r="G124" s="2" t="s">
+        <v>1068</v>
+      </c>
+      <c r="H124" s="10">
+        <v>46093.727083333331</v>
+      </c>
+    </row>
+    <row r="125" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A125" s="4">
         <v>101</v>
       </c>
@@ -4643,8 +6318,17 @@
       <c r="C125" s="5">
         <v>46092.835416666669</v>
       </c>
-    </row>
-    <row r="126" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F125" s="4">
+        <v>119</v>
+      </c>
+      <c r="G125" s="2" t="s">
+        <v>1069</v>
+      </c>
+      <c r="H125" s="10">
+        <v>46093.726388888892</v>
+      </c>
+    </row>
+    <row r="126" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A126" s="4">
         <v>102</v>
       </c>
@@ -4654,8 +6338,17 @@
       <c r="C126" s="5">
         <v>46092.833333333336</v>
       </c>
-    </row>
-    <row r="127" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F126" s="4">
+        <v>120</v>
+      </c>
+      <c r="G126" s="2" t="s">
+        <v>1070</v>
+      </c>
+      <c r="H126" s="10">
+        <v>46093.724305555559</v>
+      </c>
+    </row>
+    <row r="127" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A127" s="4">
         <v>103</v>
       </c>
@@ -4665,8 +6358,17 @@
       <c r="C127" s="5">
         <v>46092.831944444442</v>
       </c>
-    </row>
-    <row r="128" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F127" s="3">
+        <v>121</v>
+      </c>
+      <c r="G127" s="1" t="s">
+        <v>1071</v>
+      </c>
+      <c r="H127" s="10">
+        <v>46093.723611111112</v>
+      </c>
+    </row>
+    <row r="128" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A128" s="4">
         <v>104</v>
       </c>
@@ -4676,8 +6378,17 @@
       <c r="C128" s="5">
         <v>46092.830555555556</v>
       </c>
-    </row>
-    <row r="129" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F128" s="4">
+        <v>122</v>
+      </c>
+      <c r="G128" s="2" t="s">
+        <v>1072</v>
+      </c>
+      <c r="H128" s="10">
+        <v>46093.723611111112</v>
+      </c>
+    </row>
+    <row r="129" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A129" s="4">
         <v>105</v>
       </c>
@@ -4687,8 +6398,17 @@
       <c r="C129" s="5">
         <v>46092.829861111109</v>
       </c>
-    </row>
-    <row r="130" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F129" s="4">
+        <v>123</v>
+      </c>
+      <c r="G129" s="2" t="s">
+        <v>1073</v>
+      </c>
+      <c r="H129" s="10">
+        <v>46093.722222222219</v>
+      </c>
+    </row>
+    <row r="130" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A130" s="4">
         <v>106</v>
       </c>
@@ -4698,8 +6418,17 @@
       <c r="C130" s="5">
         <v>46092.827777777777</v>
       </c>
-    </row>
-    <row r="131" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F130" s="4">
+        <v>124</v>
+      </c>
+      <c r="G130" s="2" t="s">
+        <v>1074</v>
+      </c>
+      <c r="H130" s="10">
+        <v>46093.722222222219</v>
+      </c>
+    </row>
+    <row r="131" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A131" s="4">
         <v>107</v>
       </c>
@@ -4709,8 +6438,17 @@
       <c r="C131" s="5">
         <v>46092.826388888891</v>
       </c>
-    </row>
-    <row r="132" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F131" s="4">
+        <v>125</v>
+      </c>
+      <c r="G131" s="2" t="s">
+        <v>1075</v>
+      </c>
+      <c r="H131" s="10">
+        <v>46093.72152777778</v>
+      </c>
+    </row>
+    <row r="132" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A132" s="4">
         <v>108</v>
       </c>
@@ -4720,8 +6458,17 @@
       <c r="C132" s="5">
         <v>46092.822916666664</v>
       </c>
-    </row>
-    <row r="133" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F132" s="4">
+        <v>126</v>
+      </c>
+      <c r="G132" s="2" t="s">
+        <v>1076</v>
+      </c>
+      <c r="H132" s="10">
+        <v>46093.720833333333</v>
+      </c>
+    </row>
+    <row r="133" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A133" s="3">
         <v>109</v>
       </c>
@@ -4731,8 +6478,17 @@
       <c r="C133" s="5">
         <v>46092.822222222225</v>
       </c>
-    </row>
-    <row r="134" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F133" s="4">
+        <v>127</v>
+      </c>
+      <c r="G133" s="2" t="s">
+        <v>1077</v>
+      </c>
+      <c r="H133" s="10">
+        <v>46093.720138888886</v>
+      </c>
+    </row>
+    <row r="134" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A134" s="4">
         <v>110</v>
       </c>
@@ -4742,8 +6498,17 @@
       <c r="C134" s="5">
         <v>46092.822222222225</v>
       </c>
-    </row>
-    <row r="135" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F134" s="4">
+        <v>128</v>
+      </c>
+      <c r="G134" s="2" t="s">
+        <v>1078</v>
+      </c>
+      <c r="H134" s="10">
+        <v>46093.718055555553</v>
+      </c>
+    </row>
+    <row r="135" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A135" s="4">
         <v>111</v>
       </c>
@@ -4753,8 +6518,17 @@
       <c r="C135" s="5">
         <v>46092.820833333331</v>
       </c>
-    </row>
-    <row r="136" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F135" s="4">
+        <v>129</v>
+      </c>
+      <c r="G135" s="2" t="s">
+        <v>1079</v>
+      </c>
+      <c r="H135" s="10">
+        <v>46093.71597222222</v>
+      </c>
+    </row>
+    <row r="136" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A136" s="4">
         <v>112</v>
       </c>
@@ -4764,8 +6538,17 @@
       <c r="C136" s="5">
         <v>46092.820833333331</v>
       </c>
-    </row>
-    <row r="137" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F136" s="4">
+        <v>130</v>
+      </c>
+      <c r="G136" s="2" t="s">
+        <v>1080</v>
+      </c>
+      <c r="H136" s="10">
+        <v>46093.714583333334</v>
+      </c>
+    </row>
+    <row r="137" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A137" s="4">
         <v>113</v>
       </c>
@@ -4775,8 +6558,17 @@
       <c r="C137" s="5">
         <v>46092.820138888892</v>
       </c>
-    </row>
-    <row r="138" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F137" s="4">
+        <v>131</v>
+      </c>
+      <c r="G137" s="2" t="s">
+        <v>1081</v>
+      </c>
+      <c r="H137" s="10">
+        <v>46093.713888888888</v>
+      </c>
+    </row>
+    <row r="138" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A138" s="4">
         <v>114</v>
       </c>
@@ -4786,8 +6578,17 @@
       <c r="C138" s="5">
         <v>46092.819444444445</v>
       </c>
-    </row>
-    <row r="139" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F138" s="4">
+        <v>132</v>
+      </c>
+      <c r="G138" s="2" t="s">
+        <v>1082</v>
+      </c>
+      <c r="H138" s="10">
+        <v>46093.712500000001</v>
+      </c>
+    </row>
+    <row r="139" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A139" s="4">
         <v>115</v>
       </c>
@@ -4797,8 +6598,17 @@
       <c r="C139" s="5">
         <v>46092.818749999999</v>
       </c>
-    </row>
-    <row r="140" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F139" s="3">
+        <v>133</v>
+      </c>
+      <c r="G139" s="1" t="s">
+        <v>1083</v>
+      </c>
+      <c r="H139" s="10">
+        <v>46093.712500000001</v>
+      </c>
+    </row>
+    <row r="140" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A140" s="4">
         <v>116</v>
       </c>
@@ -4808,8 +6618,17 @@
       <c r="C140" s="5">
         <v>46092.818055555559</v>
       </c>
-    </row>
-    <row r="141" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F140" s="4">
+        <v>134</v>
+      </c>
+      <c r="G140" s="2" t="s">
+        <v>1084</v>
+      </c>
+      <c r="H140" s="10">
+        <v>46093.711111111108</v>
+      </c>
+    </row>
+    <row r="141" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A141" s="4">
         <v>117</v>
       </c>
@@ -4819,8 +6638,17 @@
       <c r="C141" s="5">
         <v>46092.817361111112</v>
       </c>
-    </row>
-    <row r="142" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F141" s="4">
+        <v>135</v>
+      </c>
+      <c r="G141" s="2" t="s">
+        <v>1085</v>
+      </c>
+      <c r="H141" s="10">
+        <v>46093.709722222222</v>
+      </c>
+    </row>
+    <row r="142" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A142" s="4">
         <v>118</v>
       </c>
@@ -4830,8 +6658,17 @@
       <c r="C142" s="5">
         <v>46092.817361111112</v>
       </c>
-    </row>
-    <row r="143" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F142" s="4">
+        <v>136</v>
+      </c>
+      <c r="G142" s="2" t="s">
+        <v>1086</v>
+      </c>
+      <c r="H142" s="10">
+        <v>46093.706944444442</v>
+      </c>
+    </row>
+    <row r="143" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A143" s="4">
         <v>119</v>
       </c>
@@ -4841,8 +6678,17 @@
       <c r="C143" s="5">
         <v>46092.816666666666</v>
       </c>
-    </row>
-    <row r="144" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F143" s="4">
+        <v>137</v>
+      </c>
+      <c r="G143" s="2" t="s">
+        <v>1087</v>
+      </c>
+      <c r="H143" s="10">
+        <v>46093.706250000003</v>
+      </c>
+    </row>
+    <row r="144" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A144" s="4">
         <v>120</v>
       </c>
@@ -4852,8 +6698,17 @@
       <c r="C144" s="5">
         <v>46092.813888888886</v>
       </c>
-    </row>
-    <row r="145" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F144" s="4">
+        <v>138</v>
+      </c>
+      <c r="G144" s="2" t="s">
+        <v>1088</v>
+      </c>
+      <c r="H144" s="10">
+        <v>46093.706250000003</v>
+      </c>
+    </row>
+    <row r="145" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A145" s="3">
         <v>121</v>
       </c>
@@ -4863,8 +6718,17 @@
       <c r="C145" s="5">
         <v>46092.8125</v>
       </c>
-    </row>
-    <row r="146" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F145" s="4">
+        <v>139</v>
+      </c>
+      <c r="G145" s="2" t="s">
+        <v>1089</v>
+      </c>
+      <c r="H145" s="10">
+        <v>46093.706250000003</v>
+      </c>
+    </row>
+    <row r="146" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A146" s="4">
         <v>122</v>
       </c>
@@ -4874,8 +6738,17 @@
       <c r="C146" s="5">
         <v>46092.8125</v>
       </c>
-    </row>
-    <row r="147" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F146" s="4">
+        <v>140</v>
+      </c>
+      <c r="G146" s="2" t="s">
+        <v>1090</v>
+      </c>
+      <c r="H146" s="10">
+        <v>46093.705555555556</v>
+      </c>
+    </row>
+    <row r="147" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A147" s="4">
         <v>123</v>
       </c>
@@ -4885,8 +6758,17 @@
       <c r="C147" s="5">
         <v>46092.80972222222</v>
       </c>
-    </row>
-    <row r="148" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F147" s="4">
+        <v>141</v>
+      </c>
+      <c r="G147" s="2" t="s">
+        <v>1091</v>
+      </c>
+      <c r="H147" s="10">
+        <v>46093.705555555556</v>
+      </c>
+    </row>
+    <row r="148" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A148" s="4">
         <v>124</v>
       </c>
@@ -4896,8 +6778,17 @@
       <c r="C148" s="5">
         <v>46092.80972222222</v>
       </c>
-    </row>
-    <row r="149" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F148" s="4">
+        <v>142</v>
+      </c>
+      <c r="G148" s="2" t="s">
+        <v>1092</v>
+      </c>
+      <c r="H148" s="10">
+        <v>46093.705555555556</v>
+      </c>
+    </row>
+    <row r="149" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A149" s="4">
         <v>125</v>
       </c>
@@ -4907,8 +6798,17 @@
       <c r="C149" s="5">
         <v>46092.809027777781</v>
       </c>
-    </row>
-    <row r="150" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F149" s="4">
+        <v>143</v>
+      </c>
+      <c r="G149" s="2" t="s">
+        <v>1093</v>
+      </c>
+      <c r="H149" s="10">
+        <v>46093.704861111109</v>
+      </c>
+    </row>
+    <row r="150" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A150" s="4">
         <v>126</v>
       </c>
@@ -4918,8 +6818,17 @@
       <c r="C150" s="5">
         <v>46092.808333333334</v>
       </c>
-    </row>
-    <row r="151" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F150" s="4">
+        <v>144</v>
+      </c>
+      <c r="G150" s="2" t="s">
+        <v>1094</v>
+      </c>
+      <c r="H150" s="10">
+        <v>46093.70208333333</v>
+      </c>
+    </row>
+    <row r="151" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A151" s="4">
         <v>127</v>
       </c>
@@ -4929,8 +6838,17 @@
       <c r="C151" s="5">
         <v>46092.806944444441</v>
       </c>
-    </row>
-    <row r="152" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F151" s="3">
+        <v>145</v>
+      </c>
+      <c r="G151" s="1" t="s">
+        <v>1095</v>
+      </c>
+      <c r="H151" s="10">
+        <v>46093.70208333333</v>
+      </c>
+    </row>
+    <row r="152" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A152" s="4">
         <v>128</v>
       </c>
@@ -4940,8 +6858,17 @@
       <c r="C152" s="5">
         <v>46092.806944444441</v>
       </c>
-    </row>
-    <row r="153" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F152" s="4">
+        <v>146</v>
+      </c>
+      <c r="G152" s="2" t="s">
+        <v>1096</v>
+      </c>
+      <c r="H152" s="10">
+        <v>46093.701388888891</v>
+      </c>
+    </row>
+    <row r="153" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A153" s="4">
         <v>129</v>
       </c>
@@ -4951,8 +6878,17 @@
       <c r="C153" s="5">
         <v>46092.806944444441</v>
       </c>
-    </row>
-    <row r="154" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F153" s="4">
+        <v>147</v>
+      </c>
+      <c r="G153" s="2" t="s">
+        <v>1097</v>
+      </c>
+      <c r="H153" s="10">
+        <v>46093.701388888891</v>
+      </c>
+    </row>
+    <row r="154" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A154" s="4">
         <v>130</v>
       </c>
@@ -4962,8 +6898,17 @@
       <c r="C154" s="5">
         <v>46092.806250000001</v>
       </c>
-    </row>
-    <row r="155" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F154" s="4">
+        <v>148</v>
+      </c>
+      <c r="G154" s="2" t="s">
+        <v>1098</v>
+      </c>
+      <c r="H154" s="10">
+        <v>46093.699305555558</v>
+      </c>
+    </row>
+    <row r="155" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A155" s="4">
         <v>131</v>
       </c>
@@ -4973,8 +6918,17 @@
       <c r="C155" s="5">
         <v>46092.806250000001</v>
       </c>
-    </row>
-    <row r="156" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F155" s="4">
+        <v>149</v>
+      </c>
+      <c r="G155" s="2" t="s">
+        <v>1099</v>
+      </c>
+      <c r="H155" s="10">
+        <v>46093.698611111111</v>
+      </c>
+    </row>
+    <row r="156" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A156" s="4">
         <v>132</v>
       </c>
@@ -4984,8 +6938,17 @@
       <c r="C156" s="5">
         <v>46092.805555555555</v>
       </c>
-    </row>
-    <row r="157" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F156" s="4">
+        <v>150</v>
+      </c>
+      <c r="G156" s="2" t="s">
+        <v>1100</v>
+      </c>
+      <c r="H156" s="10">
+        <v>46093.697916666664</v>
+      </c>
+    </row>
+    <row r="157" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A157" s="3">
         <v>133</v>
       </c>
@@ -4995,8 +6958,17 @@
       <c r="C157" s="5">
         <v>46092.804861111108</v>
       </c>
-    </row>
-    <row r="158" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F157" s="4">
+        <v>151</v>
+      </c>
+      <c r="G157" s="2" t="s">
+        <v>1101</v>
+      </c>
+      <c r="H157" s="10">
+        <v>46093.697222222225</v>
+      </c>
+    </row>
+    <row r="158" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A158" s="4">
         <v>134</v>
       </c>
@@ -5006,8 +6978,17 @@
       <c r="C158" s="5">
         <v>46092.804861111108</v>
       </c>
-    </row>
-    <row r="159" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F158" s="4">
+        <v>152</v>
+      </c>
+      <c r="G158" s="2" t="s">
+        <v>1102</v>
+      </c>
+      <c r="H158" s="10">
+        <v>46093.695833333331</v>
+      </c>
+    </row>
+    <row r="159" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A159" s="4">
         <v>135</v>
       </c>
@@ -5017,8 +6998,17 @@
       <c r="C159" s="5">
         <v>46092.804861111108</v>
       </c>
-    </row>
-    <row r="160" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F159" s="4">
+        <v>153</v>
+      </c>
+      <c r="G159" s="2" t="s">
+        <v>1103</v>
+      </c>
+      <c r="H159" s="10">
+        <v>46093.695833333331</v>
+      </c>
+    </row>
+    <row r="160" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A160" s="4">
         <v>136</v>
       </c>
@@ -5028,8 +7018,17 @@
       <c r="C160" s="5">
         <v>46092.804166666669</v>
       </c>
-    </row>
-    <row r="161" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F160" s="4">
+        <v>154</v>
+      </c>
+      <c r="G160" s="2" t="s">
+        <v>1104</v>
+      </c>
+      <c r="H160" s="10">
+        <v>46093.693749999999</v>
+      </c>
+    </row>
+    <row r="161" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A161" s="4">
         <v>137</v>
       </c>
@@ -5039,8 +7038,17 @@
       <c r="C161" s="5">
         <v>46092.804166666669</v>
       </c>
-    </row>
-    <row r="162" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F161" s="4">
+        <v>155</v>
+      </c>
+      <c r="G161" s="2" t="s">
+        <v>1105</v>
+      </c>
+      <c r="H161" s="10">
+        <v>46093.693749999999</v>
+      </c>
+    </row>
+    <row r="162" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A162" s="4">
         <v>138</v>
       </c>
@@ -5050,8 +7058,17 @@
       <c r="C162" s="5">
         <v>46092.802777777775</v>
       </c>
-    </row>
-    <row r="163" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F162" s="4">
+        <v>156</v>
+      </c>
+      <c r="G162" s="2" t="s">
+        <v>1106</v>
+      </c>
+      <c r="H162" s="10">
+        <v>46093.691666666666</v>
+      </c>
+    </row>
+    <row r="163" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A163" s="4">
         <v>139</v>
       </c>
@@ -5061,8 +7078,17 @@
       <c r="C163" s="5">
         <v>46092.802777777775</v>
       </c>
-    </row>
-    <row r="164" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F163" s="3">
+        <v>157</v>
+      </c>
+      <c r="G163" s="1" t="s">
+        <v>1107</v>
+      </c>
+      <c r="H163" s="10">
+        <v>46093.691666666666</v>
+      </c>
+    </row>
+    <row r="164" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A164" s="4">
         <v>140</v>
       </c>
@@ -5072,8 +7098,17 @@
       <c r="C164" s="5">
         <v>46092.802083333336</v>
       </c>
-    </row>
-    <row r="165" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F164" s="4">
+        <v>158</v>
+      </c>
+      <c r="G164" s="2" t="s">
+        <v>1108</v>
+      </c>
+      <c r="H164" s="10">
+        <v>46093.69027777778</v>
+      </c>
+    </row>
+    <row r="165" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A165" s="4">
         <v>141</v>
       </c>
@@ -5083,8 +7118,17 @@
       <c r="C165" s="5">
         <v>46092.802083333336</v>
       </c>
-    </row>
-    <row r="166" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F165" s="4">
+        <v>159</v>
+      </c>
+      <c r="G165" s="2" t="s">
+        <v>1109</v>
+      </c>
+      <c r="H165" s="10">
+        <v>46093.69027777778</v>
+      </c>
+    </row>
+    <row r="166" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A166" s="4">
         <v>142</v>
       </c>
@@ -5094,8 +7138,17 @@
       <c r="C166" s="5">
         <v>46092.800694444442</v>
       </c>
-    </row>
-    <row r="167" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F166" s="4">
+        <v>160</v>
+      </c>
+      <c r="G166" s="2" t="s">
+        <v>1110</v>
+      </c>
+      <c r="H166" s="10">
+        <v>46093.689583333333</v>
+      </c>
+    </row>
+    <row r="167" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A167" s="4">
         <v>143</v>
       </c>
@@ -5105,8 +7158,17 @@
       <c r="C167" s="5">
         <v>46092.800000000003</v>
       </c>
-    </row>
-    <row r="168" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F167" s="4">
+        <v>161</v>
+      </c>
+      <c r="G167" s="2" t="s">
+        <v>1111</v>
+      </c>
+      <c r="H167" s="10">
+        <v>46093.688194444447</v>
+      </c>
+    </row>
+    <row r="168" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A168" s="4">
         <v>144</v>
       </c>
@@ -5116,8 +7178,17 @@
       <c r="C168" s="5">
         <v>46092.800000000003</v>
       </c>
-    </row>
-    <row r="169" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F168" s="4">
+        <v>162</v>
+      </c>
+      <c r="G168" s="2" t="s">
+        <v>1112</v>
+      </c>
+      <c r="H168" s="10">
+        <v>46093.6875</v>
+      </c>
+    </row>
+    <row r="169" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A169" s="3">
         <v>145</v>
       </c>
@@ -5127,8 +7198,17 @@
       <c r="C169" s="5">
         <v>46092.800000000003</v>
       </c>
-    </row>
-    <row r="170" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F169" s="4">
+        <v>163</v>
+      </c>
+      <c r="G169" s="2" t="s">
+        <v>1113</v>
+      </c>
+      <c r="H169" s="10">
+        <v>46093.686111111114</v>
+      </c>
+    </row>
+    <row r="170" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A170" s="4">
         <v>146</v>
       </c>
@@ -5138,8 +7218,17 @@
       <c r="C170" s="5">
         <v>46092.798611111109</v>
       </c>
-    </row>
-    <row r="171" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F170" s="4">
+        <v>164</v>
+      </c>
+      <c r="G170" s="2" t="s">
+        <v>1114</v>
+      </c>
+      <c r="H170" s="10">
+        <v>46093.683333333334</v>
+      </c>
+    </row>
+    <row r="171" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A171" s="4">
         <v>147</v>
       </c>
@@ -5149,8 +7238,17 @@
       <c r="C171" s="5">
         <v>46092.79791666667</v>
       </c>
-    </row>
-    <row r="172" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F171" s="4">
+        <v>165</v>
+      </c>
+      <c r="G171" s="2" t="s">
+        <v>1115</v>
+      </c>
+      <c r="H171" s="10">
+        <v>46093.682638888888</v>
+      </c>
+    </row>
+    <row r="172" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A172" s="4">
         <v>148</v>
       </c>
@@ -5160,8 +7258,17 @@
       <c r="C172" s="5">
         <v>46092.79791666667</v>
       </c>
-    </row>
-    <row r="173" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F172" s="4">
+        <v>166</v>
+      </c>
+      <c r="G172" s="2" t="s">
+        <v>1116</v>
+      </c>
+      <c r="H172" s="10">
+        <v>46093.679861111108</v>
+      </c>
+    </row>
+    <row r="173" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A173" s="4">
         <v>149</v>
       </c>
@@ -5171,8 +7278,17 @@
       <c r="C173" s="5">
         <v>46092.79791666667</v>
       </c>
-    </row>
-    <row r="174" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F173" s="4">
+        <v>167</v>
+      </c>
+      <c r="G173" s="2" t="s">
+        <v>1117</v>
+      </c>
+      <c r="H173" s="10">
+        <v>46093.679861111108</v>
+      </c>
+    </row>
+    <row r="174" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A174" s="4">
         <v>150</v>
       </c>
@@ -5182,8 +7298,17 @@
       <c r="C174" s="5">
         <v>46092.797222222223</v>
       </c>
-    </row>
-    <row r="175" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F174" s="4">
+        <v>168</v>
+      </c>
+      <c r="G174" s="2" t="s">
+        <v>1118</v>
+      </c>
+      <c r="H174" s="10">
+        <v>46093.673611111109</v>
+      </c>
+    </row>
+    <row r="175" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A175" s="4">
         <v>151</v>
       </c>
@@ -5193,8 +7318,17 @@
       <c r="C175" s="5">
         <v>46092.797222222223</v>
       </c>
-    </row>
-    <row r="176" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F175" s="3">
+        <v>169</v>
+      </c>
+      <c r="G175" s="1" t="s">
+        <v>1119</v>
+      </c>
+      <c r="H175" s="10">
+        <v>46093.670138888891</v>
+      </c>
+    </row>
+    <row r="176" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A176" s="4">
         <v>152</v>
       </c>
@@ -5204,8 +7338,17 @@
       <c r="C176" s="5">
         <v>46092.796527777777</v>
       </c>
-    </row>
-    <row r="177" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F176" s="4">
+        <v>170</v>
+      </c>
+      <c r="G176" s="2" t="s">
+        <v>1120</v>
+      </c>
+      <c r="H176" s="10">
+        <v>46093.669444444444</v>
+      </c>
+    </row>
+    <row r="177" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A177" s="4">
         <v>153</v>
       </c>
@@ -5215,8 +7358,17 @@
       <c r="C177" s="5">
         <v>46092.796527777777</v>
       </c>
-    </row>
-    <row r="178" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F177" s="4">
+        <v>171</v>
+      </c>
+      <c r="G177" s="2" t="s">
+        <v>1121</v>
+      </c>
+      <c r="H177" s="10">
+        <v>46093.668749999997</v>
+      </c>
+    </row>
+    <row r="178" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A178" s="4">
         <v>154</v>
       </c>
@@ -5226,8 +7378,17 @@
       <c r="C178" s="5">
         <v>46092.79583333333</v>
       </c>
-    </row>
-    <row r="179" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F178" s="4">
+        <v>172</v>
+      </c>
+      <c r="G178" s="2" t="s">
+        <v>1122</v>
+      </c>
+      <c r="H178" s="10">
+        <v>46093.668055555558</v>
+      </c>
+    </row>
+    <row r="179" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A179" s="4">
         <v>155</v>
       </c>
@@ -5237,8 +7398,17 @@
       <c r="C179" s="5">
         <v>46092.79583333333</v>
       </c>
-    </row>
-    <row r="180" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F179" s="4">
+        <v>173</v>
+      </c>
+      <c r="G179" s="2" t="s">
+        <v>1123</v>
+      </c>
+      <c r="H179" s="10">
+        <v>46093.667361111111</v>
+      </c>
+    </row>
+    <row r="180" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A180" s="4">
         <v>156</v>
       </c>
@@ -5248,8 +7418,17 @@
       <c r="C180" s="5">
         <v>46092.794444444444</v>
       </c>
-    </row>
-    <row r="181" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F180" s="4">
+        <v>174</v>
+      </c>
+      <c r="G180" s="2" t="s">
+        <v>1124</v>
+      </c>
+      <c r="H180" s="10">
+        <v>46093.667361111111</v>
+      </c>
+    </row>
+    <row r="181" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A181" s="3">
         <v>157</v>
       </c>
@@ -5259,8 +7438,17 @@
       <c r="C181" s="5">
         <v>46092.793749999997</v>
       </c>
-    </row>
-    <row r="182" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F181" s="4">
+        <v>175</v>
+      </c>
+      <c r="G181" s="2" t="s">
+        <v>1125</v>
+      </c>
+      <c r="H181" s="10">
+        <v>46093.666666666664</v>
+      </c>
+    </row>
+    <row r="182" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A182" s="4">
         <v>158</v>
       </c>
@@ -5270,8 +7458,17 @@
       <c r="C182" s="5">
         <v>46092.793749999997</v>
       </c>
-    </row>
-    <row r="183" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F182" s="4">
+        <v>176</v>
+      </c>
+      <c r="G182" s="2" t="s">
+        <v>1126</v>
+      </c>
+      <c r="H182" s="10">
+        <v>46093.665277777778</v>
+      </c>
+    </row>
+    <row r="183" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A183" s="4">
         <v>159</v>
       </c>
@@ -5281,8 +7478,17 @@
       <c r="C183" s="5">
         <v>46092.793749999997</v>
       </c>
-    </row>
-    <row r="184" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F183" s="4">
+        <v>177</v>
+      </c>
+      <c r="G183" s="2" t="s">
+        <v>1127</v>
+      </c>
+      <c r="H183" s="10">
+        <v>46093.665277777778</v>
+      </c>
+    </row>
+    <row r="184" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A184" s="4">
         <v>160</v>
       </c>
@@ -5292,8 +7498,17 @@
       <c r="C184" s="5">
         <v>46092.792361111111</v>
       </c>
-    </row>
-    <row r="185" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F184" s="4">
+        <v>178</v>
+      </c>
+      <c r="G184" s="2" t="s">
+        <v>1128</v>
+      </c>
+      <c r="H184" s="10">
+        <v>46093.665277777778</v>
+      </c>
+    </row>
+    <row r="185" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A185" s="4">
         <v>161</v>
       </c>
@@ -5303,8 +7518,17 @@
       <c r="C185" s="5">
         <v>46092.792361111111</v>
       </c>
-    </row>
-    <row r="186" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F185" s="4">
+        <v>179</v>
+      </c>
+      <c r="G185" s="2" t="s">
+        <v>1129</v>
+      </c>
+      <c r="H185" s="10">
+        <v>46093.664583333331</v>
+      </c>
+    </row>
+    <row r="186" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A186" s="4">
         <v>162</v>
       </c>
@@ -5314,8 +7538,17 @@
       <c r="C186" s="5">
         <v>46092.791666666664</v>
       </c>
-    </row>
-    <row r="187" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F186" s="4">
+        <v>180</v>
+      </c>
+      <c r="G186" s="2" t="s">
+        <v>1130</v>
+      </c>
+      <c r="H186" s="10">
+        <v>46093.664583333331</v>
+      </c>
+    </row>
+    <row r="187" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A187" s="4">
         <v>163</v>
       </c>
@@ -5325,8 +7558,17 @@
       <c r="C187" s="5">
         <v>46092.790277777778</v>
       </c>
-    </row>
-    <row r="188" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F187" s="3">
+        <v>181</v>
+      </c>
+      <c r="G187" s="1" t="s">
+        <v>1131</v>
+      </c>
+      <c r="H187" s="10">
+        <v>46093.663888888892</v>
+      </c>
+    </row>
+    <row r="188" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A188" s="4">
         <v>164</v>
       </c>
@@ -5336,8 +7578,17 @@
       <c r="C188" s="5">
         <v>46092.788194444445</v>
       </c>
-    </row>
-    <row r="189" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F188" s="4">
+        <v>182</v>
+      </c>
+      <c r="G188" s="2" t="s">
+        <v>1132</v>
+      </c>
+      <c r="H188" s="10">
+        <v>46093.661805555559</v>
+      </c>
+    </row>
+    <row r="189" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A189" s="4">
         <v>165</v>
       </c>
@@ -5347,8 +7598,17 @@
       <c r="C189" s="5">
         <v>46092.788194444445</v>
       </c>
-    </row>
-    <row r="190" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F189" s="4">
+        <v>183</v>
+      </c>
+      <c r="G189" s="2" t="s">
+        <v>1133</v>
+      </c>
+      <c r="H189" s="10">
+        <v>46093.661111111112</v>
+      </c>
+    </row>
+    <row r="190" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A190" s="4">
         <v>166</v>
       </c>
@@ -5358,8 +7618,17 @@
       <c r="C190" s="5">
         <v>46092.787499999999</v>
       </c>
-    </row>
-    <row r="191" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F190" s="4">
+        <v>184</v>
+      </c>
+      <c r="G190" s="2" t="s">
+        <v>1134</v>
+      </c>
+      <c r="H190" s="10">
+        <v>46093.659722222219</v>
+      </c>
+    </row>
+    <row r="191" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A191" s="4">
         <v>167</v>
       </c>
@@ -5369,8 +7638,17 @@
       <c r="C191" s="5">
         <v>46092.785416666666</v>
       </c>
-    </row>
-    <row r="192" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F191" s="4">
+        <v>185</v>
+      </c>
+      <c r="G191" s="2" t="s">
+        <v>1135</v>
+      </c>
+      <c r="H191" s="10">
+        <v>46093.657638888886</v>
+      </c>
+    </row>
+    <row r="192" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A192" s="4">
         <v>168</v>
       </c>
@@ -5380,8 +7658,17 @@
       <c r="C192" s="5">
         <v>46092.785416666666</v>
       </c>
-    </row>
-    <row r="193" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F192" s="4">
+        <v>186</v>
+      </c>
+      <c r="G192" s="2" t="s">
+        <v>1136</v>
+      </c>
+      <c r="H192" s="10">
+        <v>46093.656944444447</v>
+      </c>
+    </row>
+    <row r="193" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A193" s="3">
         <v>169</v>
       </c>
@@ -5391,8 +7678,17 @@
       <c r="C193" s="5">
         <v>46092.784722222219</v>
       </c>
-    </row>
-    <row r="194" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F193" s="4">
+        <v>187</v>
+      </c>
+      <c r="G193" s="2" t="s">
+        <v>1137</v>
+      </c>
+      <c r="H193" s="10">
+        <v>46093.655555555553</v>
+      </c>
+    </row>
+    <row r="194" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A194" s="4">
         <v>170</v>
       </c>
@@ -5402,8 +7698,17 @@
       <c r="C194" s="5">
         <v>46092.784722222219</v>
       </c>
-    </row>
-    <row r="195" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F194" s="4">
+        <v>188</v>
+      </c>
+      <c r="G194" s="2" t="s">
+        <v>1138</v>
+      </c>
+      <c r="H194" s="10">
+        <v>46093.654861111114</v>
+      </c>
+    </row>
+    <row r="195" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A195" s="4">
         <v>171</v>
       </c>
@@ -5413,8 +7718,17 @@
       <c r="C195" s="5">
         <v>46092.784722222219</v>
       </c>
-    </row>
-    <row r="196" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F195" s="4">
+        <v>189</v>
+      </c>
+      <c r="G195" s="2" t="s">
+        <v>1139</v>
+      </c>
+      <c r="H195" s="10">
+        <v>46093.654861111114</v>
+      </c>
+    </row>
+    <row r="196" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A196" s="4">
         <v>172</v>
       </c>
@@ -5424,8 +7738,17 @@
       <c r="C196" s="5">
         <v>46092.78402777778</v>
       </c>
-    </row>
-    <row r="197" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F196" s="4">
+        <v>190</v>
+      </c>
+      <c r="G196" s="2" t="s">
+        <v>1140</v>
+      </c>
+      <c r="H196" s="10">
+        <v>46093.654166666667</v>
+      </c>
+    </row>
+    <row r="197" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A197" s="4">
         <v>173</v>
       </c>
@@ -5435,8 +7758,17 @@
       <c r="C197" s="5">
         <v>46092.78402777778</v>
       </c>
-    </row>
-    <row r="198" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F197" s="4">
+        <v>191</v>
+      </c>
+      <c r="G197" s="2" t="s">
+        <v>1141</v>
+      </c>
+      <c r="H197" s="10">
+        <v>46093.652777777781</v>
+      </c>
+    </row>
+    <row r="198" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A198" s="4">
         <v>174</v>
       </c>
@@ -5446,8 +7778,17 @@
       <c r="C198" s="5">
         <v>46092.783333333333</v>
       </c>
-    </row>
-    <row r="199" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F198" s="4">
+        <v>192</v>
+      </c>
+      <c r="G198" s="2" t="s">
+        <v>1142</v>
+      </c>
+      <c r="H198" s="10">
+        <v>46093.652777777781</v>
+      </c>
+    </row>
+    <row r="199" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A199" s="4">
         <v>175</v>
       </c>
@@ -5457,8 +7798,17 @@
       <c r="C199" s="5">
         <v>46092.783333333333</v>
       </c>
-    </row>
-    <row r="200" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F199" s="3">
+        <v>193</v>
+      </c>
+      <c r="G199" s="1" t="s">
+        <v>1143</v>
+      </c>
+      <c r="H199" s="10">
+        <v>46093.652083333334</v>
+      </c>
+    </row>
+    <row r="200" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A200" s="4">
         <v>176</v>
       </c>
@@ -5468,8 +7818,17 @@
       <c r="C200" s="5">
         <v>46092.783333333333</v>
       </c>
-    </row>
-    <row r="201" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F200" s="4">
+        <v>194</v>
+      </c>
+      <c r="G200" s="2" t="s">
+        <v>1144</v>
+      </c>
+      <c r="H200" s="10">
+        <v>46093.651388888888</v>
+      </c>
+    </row>
+    <row r="201" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A201" s="4">
         <v>177</v>
       </c>
@@ -5479,8 +7838,17 @@
       <c r="C201" s="5">
         <v>46092.782638888886</v>
       </c>
-    </row>
-    <row r="202" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F201" s="4">
+        <v>195</v>
+      </c>
+      <c r="G201" s="2" t="s">
+        <v>1145</v>
+      </c>
+      <c r="H201" s="10">
+        <v>46093.650694444441</v>
+      </c>
+    </row>
+    <row r="202" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A202" s="4">
         <v>178</v>
       </c>
@@ -5490,8 +7858,17 @@
       <c r="C202" s="5">
         <v>46092.782638888886</v>
       </c>
-    </row>
-    <row r="203" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F202" s="4">
+        <v>196</v>
+      </c>
+      <c r="G202" s="2" t="s">
+        <v>1146</v>
+      </c>
+      <c r="H202" s="10">
+        <v>46093.65</v>
+      </c>
+    </row>
+    <row r="203" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A203" s="4">
         <v>179</v>
       </c>
@@ -5501,8 +7878,17 @@
       <c r="C203" s="5">
         <v>46092.781944444447</v>
       </c>
-    </row>
-    <row r="204" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F203" s="4">
+        <v>197</v>
+      </c>
+      <c r="G203" s="2" t="s">
+        <v>1147</v>
+      </c>
+      <c r="H203" s="10">
+        <v>46093.65</v>
+      </c>
+    </row>
+    <row r="204" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A204" s="4">
         <v>180</v>
       </c>
@@ -5512,8 +7898,17 @@
       <c r="C204" s="5">
         <v>46092.781944444447</v>
       </c>
-    </row>
-    <row r="205" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F204" s="4">
+        <v>198</v>
+      </c>
+      <c r="G204" s="2" t="s">
+        <v>1148</v>
+      </c>
+      <c r="H204" s="10">
+        <v>46093.649305555555</v>
+      </c>
+    </row>
+    <row r="205" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A205" s="3">
         <v>181</v>
       </c>
@@ -5523,8 +7918,17 @@
       <c r="C205" s="5">
         <v>46092.781944444447</v>
       </c>
-    </row>
-    <row r="206" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F205" s="4">
+        <v>199</v>
+      </c>
+      <c r="G205" s="2" t="s">
+        <v>1149</v>
+      </c>
+      <c r="H205" s="10">
+        <v>46093.649305555555</v>
+      </c>
+    </row>
+    <row r="206" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A206" s="4">
         <v>182</v>
       </c>
@@ -5534,8 +7938,17 @@
       <c r="C206" s="5">
         <v>46092.781944444447</v>
       </c>
-    </row>
-    <row r="207" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F206" s="4">
+        <v>200</v>
+      </c>
+      <c r="G206" s="2" t="s">
+        <v>1150</v>
+      </c>
+      <c r="H206" s="10">
+        <v>46093.647916666669</v>
+      </c>
+    </row>
+    <row r="207" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A207" s="4">
         <v>183</v>
       </c>
@@ -5545,8 +7958,17 @@
       <c r="C207" s="5">
         <v>46092.78125</v>
       </c>
-    </row>
-    <row r="208" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F207" s="4">
+        <v>201</v>
+      </c>
+      <c r="G207" s="2" t="s">
+        <v>1151</v>
+      </c>
+      <c r="H207" s="10">
+        <v>46093.647222222222</v>
+      </c>
+    </row>
+    <row r="208" spans="1:8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A208" s="4">
         <v>184</v>
       </c>
@@ -5555,6 +7977,15 @@
       </c>
       <c r="C208" s="5">
         <v>46092.780555555553</v>
+      </c>
+      <c r="F208" s="4">
+        <v>202</v>
+      </c>
+      <c r="G208" s="2" t="s">
+        <v>1152</v>
+      </c>
+      <c r="H208" s="10">
+        <v>46093.647222222222</v>
       </c>
     </row>
     <row r="209" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">

</xml_diff>